<commit_message>
Documentos de proyecto finales Capstone 2025
</commit_message>
<xml_diff>
--- a/Planilla Registro de Riesgos.xlsx
+++ b/Planilla Registro de Riesgos.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="jtX1KB5++8WR5Elw5a6ROPUHfAoJKtnXGMo428hmwqU="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="H/X6cITRqYWrMeUTnMp3lKYUt5JcZ+JxBx3ALDILhls="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="123">
   <si>
     <t>ID del Proyecto</t>
   </si>
@@ -282,7 +282,7 @@
     <t xml:space="preserve">Direccion proyecto </t>
   </si>
   <si>
-    <t>Falla de sincronización labial y facial en el avatar</t>
+    <t>Falla de sincronizaciónen el avatar</t>
   </si>
   <si>
     <t>Expresión facial</t>
@@ -316,6 +316,78 @@
   </si>
   <si>
     <t>se asegurará una carga de trabajo balanceada, se fomentará la comunicación abierta y el apoyo mutuo, y se implementarán descansos y reconocimiento de logros para mantener la motivación alta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dependencia de un inteprete de lengua de señas </t>
+  </si>
+  <si>
+    <t>Gestion de equipo</t>
+  </si>
+  <si>
+    <t>Retraso en la codificación y validación del sistema de traducción.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La dependencia de un interprete para resolver dudas presentes durante la fase del proyecto, como tambien la necesidad de orientacion </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usabilidad </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alta </t>
+  </si>
+  <si>
+    <t>ALTA</t>
+  </si>
+  <si>
+    <t>Establecer alianzas tempranas con instituciones o asociaciones especializadas</t>
+  </si>
+  <si>
+    <t>Equipo de desarrollo y empresa externa</t>
+  </si>
+  <si>
+    <t>Limitaciones en la digitalización del lenguaje hablado</t>
+  </si>
+  <si>
+    <t>Calidad del producto</t>
+  </si>
+  <si>
+    <t>Pérdida de fidelidad en la traducción y comprensión limitada</t>
+  </si>
+  <si>
+    <t>Insuficiencia de modelos entrenados o falta de base de datos robusta</t>
+  </si>
+  <si>
+    <t>Tecnología / Usabilidad</t>
+  </si>
+  <si>
+    <t>Altto</t>
+  </si>
+  <si>
+    <t>Mitigar</t>
+  </si>
+  <si>
+    <t>Entrenar modelos con corpus diverso y validado, colaboración con expertos en lengua de señas</t>
+  </si>
+  <si>
+    <t>Desfase entre el lenguaje inclusivo y la representación visual</t>
+  </si>
+  <si>
+    <t>Comunicación</t>
+  </si>
+  <si>
+    <t>Posible percepción negativa o malinterpretaciones del mensaje</t>
+  </si>
+  <si>
+    <t>Evolución del lenguaje inclusivo más rápida que su representación en señas</t>
+  </si>
+  <si>
+    <t>Comuunicacion/social</t>
+  </si>
+  <si>
+    <t>Medio</t>
+  </si>
+  <si>
+    <t>Consultas continuas con comunidades sordas y lingüistas inclusivos</t>
   </si>
 </sst>
 </file>
@@ -404,7 +476,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="18">
     <border/>
     <border>
       <left/>
@@ -516,6 +588,15 @@
       <top/>
     </border>
     <border>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <right/>
+      <bottom/>
+    </border>
+    <border>
       <left/>
       <right/>
       <bottom/>
@@ -524,7 +605,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="41">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -587,37 +668,50 @@
     <xf borderId="14" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="9" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="9" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="15" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="9" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="10" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="9" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="9" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="9" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="15" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="9" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="9" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="15" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="9" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="16" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="17" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="17" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1615,540 +1709,770 @@
       </c>
       <c r="X16" s="23"/>
     </row>
-    <row r="17" ht="12.75" customHeight="1">
-      <c r="A17" s="24"/>
-      <c r="B17" s="25"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="I17" s="25"/>
-      <c r="K17" s="25"/>
-      <c r="M17" s="25"/>
-      <c r="O17" s="25"/>
-      <c r="Q17" s="25"/>
-      <c r="S17" s="25"/>
-      <c r="U17" s="25"/>
-      <c r="V17" s="26"/>
-      <c r="W17" s="25"/>
-      <c r="X17" s="27"/>
-    </row>
-    <row r="18" ht="12.75" customHeight="1">
-      <c r="A18" s="24"/>
-      <c r="B18" s="25"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
-      <c r="I18" s="25"/>
-      <c r="K18" s="25"/>
-      <c r="M18" s="25"/>
-      <c r="O18" s="25"/>
-      <c r="Q18" s="25"/>
-      <c r="S18" s="25"/>
-      <c r="U18" s="25"/>
-      <c r="V18" s="26"/>
-      <c r="W18" s="25"/>
-      <c r="X18" s="27"/>
-    </row>
-    <row r="19" ht="84.0" customHeight="1">
-      <c r="A19" s="24"/>
-      <c r="B19" s="25"/>
-      <c r="C19" s="25"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
-      <c r="I19" s="25"/>
-      <c r="K19" s="25"/>
-      <c r="M19" s="25"/>
-      <c r="O19" s="25"/>
-      <c r="Q19" s="25"/>
-      <c r="S19" s="25"/>
-      <c r="U19" s="25"/>
-      <c r="V19" s="26"/>
-      <c r="W19" s="25"/>
-      <c r="X19" s="27"/>
-    </row>
-    <row r="20" ht="12.75" customHeight="1">
-      <c r="A20" s="24"/>
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="I20" s="25"/>
-      <c r="K20" s="25"/>
-      <c r="M20" s="25"/>
-      <c r="O20" s="25"/>
-      <c r="Q20" s="25"/>
-      <c r="S20" s="25"/>
-      <c r="U20" s="25"/>
-      <c r="V20" s="26"/>
-      <c r="W20" s="25"/>
-      <c r="X20" s="27"/>
-    </row>
-    <row r="21" ht="12.75" customHeight="1">
-      <c r="A21" s="24"/>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="I21" s="25"/>
-      <c r="K21" s="25"/>
-      <c r="M21" s="25"/>
-      <c r="O21" s="25"/>
-      <c r="Q21" s="25"/>
-      <c r="S21" s="25"/>
-      <c r="U21" s="25"/>
-      <c r="V21" s="26"/>
-      <c r="W21" s="25"/>
-      <c r="X21" s="27"/>
-    </row>
-    <row r="22" ht="12.75" customHeight="1">
-      <c r="A22" s="24"/>
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="I22" s="25"/>
-      <c r="K22" s="25"/>
-      <c r="M22" s="25"/>
-      <c r="O22" s="25"/>
-      <c r="Q22" s="25"/>
-      <c r="S22" s="25"/>
-      <c r="U22" s="25"/>
-      <c r="V22" s="26"/>
-      <c r="W22" s="25"/>
-      <c r="X22" s="27"/>
+    <row r="17" ht="60.0" customHeight="1">
+      <c r="A17" s="21"/>
+      <c r="B17" s="18">
+        <v>11.0</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="F17" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="G17" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="H17" s="13"/>
+      <c r="I17" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="J17" s="13"/>
+      <c r="K17" s="19">
+        <v>5.0</v>
+      </c>
+      <c r="L17" s="13"/>
+      <c r="M17" s="19">
+        <v>3.0</v>
+      </c>
+      <c r="N17" s="13"/>
+      <c r="O17" s="19">
+        <v>15.0</v>
+      </c>
+      <c r="P17" s="13"/>
+      <c r="Q17" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="R17" s="13"/>
+      <c r="S17" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="T17" s="13"/>
+      <c r="U17" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="V17" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="W17" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="X17" s="25"/>
+    </row>
+    <row r="18" ht="84.0" customHeight="1">
+      <c r="A18" s="21"/>
+      <c r="B18" s="18">
+        <v>13.0</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="E18" s="26" t="s">
+        <v>110</v>
+      </c>
+      <c r="F18" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="G18" s="27" t="s">
+        <v>112</v>
+      </c>
+      <c r="H18" s="28"/>
+      <c r="I18" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="J18" s="28"/>
+      <c r="K18" s="19">
+        <v>5.0</v>
+      </c>
+      <c r="L18" s="13"/>
+      <c r="M18" s="19">
+        <v>5.0</v>
+      </c>
+      <c r="N18" s="13"/>
+      <c r="O18" s="19">
+        <v>20.0</v>
+      </c>
+      <c r="P18" s="13"/>
+      <c r="Q18" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="R18" s="13"/>
+      <c r="S18" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="T18" s="13"/>
+      <c r="U18" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="V18" s="26" t="s">
+        <v>115</v>
+      </c>
+      <c r="W18" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="X18" s="25"/>
+    </row>
+    <row r="19" ht="43.5" customHeight="1">
+      <c r="A19" s="21"/>
+      <c r="B19" s="18">
+        <v>14.0</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="D19" s="26" t="s">
+        <v>117</v>
+      </c>
+      <c r="E19" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="F19" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="G19" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="H19" s="13"/>
+      <c r="I19" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="J19" s="13"/>
+      <c r="K19" s="19">
+        <v>2.0</v>
+      </c>
+      <c r="L19" s="13"/>
+      <c r="M19" s="19">
+        <v>4.0</v>
+      </c>
+      <c r="N19" s="13"/>
+      <c r="O19" s="19">
+        <v>8.0</v>
+      </c>
+      <c r="P19" s="13"/>
+      <c r="Q19" s="27" t="s">
+        <v>38</v>
+      </c>
+      <c r="R19" s="28"/>
+      <c r="S19" s="27" t="s">
+        <v>121</v>
+      </c>
+      <c r="T19" s="28"/>
+      <c r="U19" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="V19" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="W19" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="X19" s="25"/>
+    </row>
+    <row r="20" ht="60.75" customHeight="1">
+      <c r="A20" s="21"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="30"/>
+      <c r="J20" s="13"/>
+      <c r="K20" s="30"/>
+      <c r="L20" s="13"/>
+      <c r="M20" s="30"/>
+      <c r="N20" s="13"/>
+      <c r="O20" s="30"/>
+      <c r="P20" s="13"/>
+      <c r="Q20" s="30"/>
+      <c r="R20" s="13"/>
+      <c r="S20" s="30"/>
+      <c r="T20" s="13"/>
+      <c r="U20" s="29"/>
+      <c r="V20" s="31"/>
+      <c r="W20" s="29"/>
+      <c r="X20" s="25"/>
+    </row>
+    <row r="21" ht="56.25" customHeight="1">
+      <c r="A21" s="21"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="30"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="30"/>
+      <c r="J21" s="13"/>
+      <c r="K21" s="30"/>
+      <c r="L21" s="13"/>
+      <c r="M21" s="30"/>
+      <c r="N21" s="13"/>
+      <c r="O21" s="30"/>
+      <c r="P21" s="13"/>
+      <c r="Q21" s="30"/>
+      <c r="R21" s="13"/>
+      <c r="S21" s="30"/>
+      <c r="T21" s="13"/>
+      <c r="U21" s="29"/>
+      <c r="V21" s="31"/>
+      <c r="W21" s="29"/>
+      <c r="X21" s="25"/>
+    </row>
+    <row r="22" ht="72.0" customHeight="1">
+      <c r="A22" s="21"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="30"/>
+      <c r="H22" s="13"/>
+      <c r="I22" s="30"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="30"/>
+      <c r="L22" s="13"/>
+      <c r="M22" s="30"/>
+      <c r="N22" s="13"/>
+      <c r="O22" s="30"/>
+      <c r="P22" s="13"/>
+      <c r="Q22" s="30"/>
+      <c r="R22" s="13"/>
+      <c r="S22" s="30"/>
+      <c r="T22" s="13"/>
+      <c r="U22" s="29"/>
+      <c r="V22" s="31"/>
+      <c r="W22" s="29"/>
+      <c r="X22" s="25"/>
     </row>
     <row r="23" ht="12.75" customHeight="1">
-      <c r="A23" s="24"/>
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="25"/>
-      <c r="I23" s="25"/>
-      <c r="K23" s="25"/>
-      <c r="M23" s="25"/>
-      <c r="O23" s="25"/>
-      <c r="Q23" s="25"/>
-      <c r="S23" s="25"/>
-      <c r="U23" s="25"/>
-      <c r="V23" s="26"/>
-      <c r="W23" s="25"/>
-      <c r="X23" s="27"/>
+      <c r="A23" s="21"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="30"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="30"/>
+      <c r="J23" s="13"/>
+      <c r="K23" s="30"/>
+      <c r="L23" s="13"/>
+      <c r="M23" s="30"/>
+      <c r="N23" s="13"/>
+      <c r="O23" s="30"/>
+      <c r="P23" s="13"/>
+      <c r="Q23" s="30"/>
+      <c r="R23" s="13"/>
+      <c r="S23" s="30"/>
+      <c r="T23" s="13"/>
+      <c r="U23" s="29"/>
+      <c r="V23" s="31"/>
+      <c r="W23" s="29"/>
+      <c r="X23" s="25"/>
     </row>
     <row r="24" ht="12.75" customHeight="1">
-      <c r="A24" s="24"/>
-      <c r="B24" s="25"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="I24" s="25"/>
-      <c r="K24" s="25"/>
-      <c r="M24" s="25"/>
-      <c r="O24" s="25"/>
-      <c r="Q24" s="25"/>
-      <c r="S24" s="25"/>
-      <c r="U24" s="25"/>
-      <c r="V24" s="26"/>
-      <c r="W24" s="25"/>
-      <c r="X24" s="27"/>
+      <c r="A24" s="21"/>
+      <c r="B24" s="29"/>
+      <c r="C24" s="29"/>
+      <c r="D24" s="29"/>
+      <c r="E24" s="29"/>
+      <c r="F24" s="29"/>
+      <c r="G24" s="30"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="30"/>
+      <c r="J24" s="13"/>
+      <c r="K24" s="30"/>
+      <c r="L24" s="13"/>
+      <c r="M24" s="30"/>
+      <c r="N24" s="13"/>
+      <c r="O24" s="30"/>
+      <c r="P24" s="13"/>
+      <c r="Q24" s="30"/>
+      <c r="R24" s="13"/>
+      <c r="S24" s="30"/>
+      <c r="T24" s="13"/>
+      <c r="U24" s="29"/>
+      <c r="V24" s="31"/>
+      <c r="W24" s="29"/>
+      <c r="X24" s="25"/>
     </row>
     <row r="25" ht="12.75" customHeight="1">
-      <c r="A25" s="24"/>
-      <c r="B25" s="25"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="25"/>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="25"/>
-      <c r="I25" s="25"/>
-      <c r="K25" s="25"/>
-      <c r="M25" s="25"/>
-      <c r="O25" s="25"/>
-      <c r="Q25" s="25"/>
-      <c r="S25" s="25"/>
-      <c r="U25" s="25"/>
-      <c r="V25" s="26"/>
-      <c r="W25" s="25"/>
-      <c r="X25" s="27"/>
-    </row>
-    <row r="26" ht="12.75" customHeight="1">
-      <c r="A26" s="24"/>
-      <c r="B26" s="25"/>
-      <c r="C26" s="25"/>
-      <c r="D26" s="25"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="25"/>
-      <c r="I26" s="25"/>
-      <c r="K26" s="25"/>
-      <c r="M26" s="25"/>
-      <c r="O26" s="25"/>
-      <c r="Q26" s="25"/>
-      <c r="S26" s="25"/>
-      <c r="U26" s="25"/>
-      <c r="V26" s="26"/>
-      <c r="W26" s="25"/>
-      <c r="X26" s="27"/>
-    </row>
-    <row r="27" ht="58.5" customHeight="1">
-      <c r="A27" s="24"/>
-      <c r="B27" s="25"/>
-      <c r="C27" s="25"/>
-      <c r="D27" s="25"/>
-      <c r="E27" s="25"/>
-      <c r="F27" s="25"/>
-      <c r="G27" s="25"/>
-      <c r="I27" s="25"/>
-      <c r="K27" s="25"/>
-      <c r="M27" s="25"/>
-      <c r="O27" s="25"/>
-      <c r="Q27" s="25"/>
-      <c r="S27" s="25"/>
-      <c r="U27" s="25"/>
-      <c r="V27" s="26"/>
-      <c r="W27" s="25"/>
-      <c r="X27" s="27"/>
+      <c r="A25" s="21"/>
+      <c r="B25" s="29"/>
+      <c r="C25" s="29"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="29"/>
+      <c r="G25" s="30"/>
+      <c r="H25" s="13"/>
+      <c r="I25" s="30"/>
+      <c r="J25" s="13"/>
+      <c r="K25" s="30"/>
+      <c r="L25" s="13"/>
+      <c r="M25" s="30"/>
+      <c r="N25" s="13"/>
+      <c r="O25" s="30"/>
+      <c r="P25" s="13"/>
+      <c r="Q25" s="30"/>
+      <c r="R25" s="13"/>
+      <c r="S25" s="30"/>
+      <c r="T25" s="13"/>
+      <c r="U25" s="29"/>
+      <c r="V25" s="31"/>
+      <c r="W25" s="29"/>
+      <c r="X25" s="25"/>
+    </row>
+    <row r="26" ht="58.5" customHeight="1">
+      <c r="A26" s="21"/>
+      <c r="B26" s="29"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="30"/>
+      <c r="H26" s="13"/>
+      <c r="I26" s="30"/>
+      <c r="J26" s="13"/>
+      <c r="K26" s="30"/>
+      <c r="L26" s="13"/>
+      <c r="M26" s="30"/>
+      <c r="N26" s="13"/>
+      <c r="O26" s="30"/>
+      <c r="P26" s="13"/>
+      <c r="Q26" s="30"/>
+      <c r="R26" s="13"/>
+      <c r="S26" s="30"/>
+      <c r="T26" s="13"/>
+      <c r="U26" s="29"/>
+      <c r="V26" s="31"/>
+      <c r="W26" s="29"/>
+      <c r="X26" s="25"/>
+    </row>
+    <row r="27" ht="12.75" customHeight="1">
+      <c r="A27" s="21"/>
+      <c r="B27" s="29"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="13"/>
+      <c r="I27" s="30"/>
+      <c r="J27" s="13"/>
+      <c r="K27" s="30"/>
+      <c r="L27" s="13"/>
+      <c r="M27" s="30"/>
+      <c r="N27" s="13"/>
+      <c r="O27" s="30"/>
+      <c r="P27" s="13"/>
+      <c r="Q27" s="30"/>
+      <c r="R27" s="13"/>
+      <c r="S27" s="30"/>
+      <c r="T27" s="13"/>
+      <c r="U27" s="29"/>
+      <c r="V27" s="31"/>
+      <c r="W27" s="29"/>
+      <c r="X27" s="25"/>
     </row>
     <row r="28" ht="12.75" customHeight="1">
-      <c r="A28" s="24"/>
-      <c r="B28" s="25"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="25"/>
-      <c r="I28" s="25"/>
-      <c r="K28" s="25"/>
-      <c r="M28" s="25"/>
-      <c r="O28" s="25"/>
-      <c r="Q28" s="25"/>
-      <c r="S28" s="25"/>
-      <c r="U28" s="25"/>
-      <c r="V28" s="26"/>
-      <c r="W28" s="25"/>
-      <c r="X28" s="27"/>
+      <c r="A28" s="21"/>
+      <c r="B28" s="29"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="13"/>
+      <c r="I28" s="30"/>
+      <c r="J28" s="13"/>
+      <c r="K28" s="30"/>
+      <c r="L28" s="13"/>
+      <c r="M28" s="30"/>
+      <c r="N28" s="13"/>
+      <c r="O28" s="30"/>
+      <c r="P28" s="13"/>
+      <c r="Q28" s="30"/>
+      <c r="R28" s="13"/>
+      <c r="S28" s="30"/>
+      <c r="T28" s="13"/>
+      <c r="U28" s="29"/>
+      <c r="V28" s="31"/>
+      <c r="W28" s="29"/>
+      <c r="X28" s="25"/>
     </row>
     <row r="29" ht="12.75" customHeight="1">
-      <c r="A29" s="24"/>
-      <c r="B29" s="25"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="25"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="25"/>
-      <c r="G29" s="25"/>
-      <c r="I29" s="25"/>
-      <c r="K29" s="25"/>
-      <c r="M29" s="25"/>
-      <c r="O29" s="25"/>
-      <c r="Q29" s="25"/>
-      <c r="S29" s="25"/>
-      <c r="U29" s="25"/>
-      <c r="V29" s="26"/>
-      <c r="W29" s="25"/>
-      <c r="X29" s="27"/>
+      <c r="A29" s="21"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="30"/>
+      <c r="H29" s="13"/>
+      <c r="I29" s="30"/>
+      <c r="J29" s="13"/>
+      <c r="K29" s="30"/>
+      <c r="L29" s="13"/>
+      <c r="M29" s="30"/>
+      <c r="N29" s="13"/>
+      <c r="O29" s="30"/>
+      <c r="P29" s="13"/>
+      <c r="Q29" s="30"/>
+      <c r="R29" s="13"/>
+      <c r="S29" s="30"/>
+      <c r="T29" s="13"/>
+      <c r="U29" s="29"/>
+      <c r="V29" s="31"/>
+      <c r="W29" s="29"/>
+      <c r="X29" s="25"/>
     </row>
     <row r="30" ht="12.75" customHeight="1">
-      <c r="A30" s="24"/>
-      <c r="B30" s="25"/>
-      <c r="C30" s="25"/>
-      <c r="D30" s="25"/>
-      <c r="E30" s="25"/>
-      <c r="F30" s="25"/>
-      <c r="G30" s="25"/>
-      <c r="I30" s="25"/>
-      <c r="K30" s="25"/>
-      <c r="M30" s="25"/>
-      <c r="O30" s="25"/>
-      <c r="Q30" s="25"/>
-      <c r="S30" s="25"/>
-      <c r="U30" s="25"/>
-      <c r="V30" s="26"/>
-      <c r="W30" s="25"/>
-      <c r="X30" s="27"/>
+      <c r="A30" s="21"/>
+      <c r="B30" s="29"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="29"/>
+      <c r="F30" s="29"/>
+      <c r="G30" s="30"/>
+      <c r="H30" s="13"/>
+      <c r="I30" s="30"/>
+      <c r="J30" s="13"/>
+      <c r="K30" s="30"/>
+      <c r="L30" s="13"/>
+      <c r="M30" s="30"/>
+      <c r="N30" s="13"/>
+      <c r="O30" s="30"/>
+      <c r="P30" s="13"/>
+      <c r="Q30" s="30"/>
+      <c r="R30" s="13"/>
+      <c r="S30" s="30"/>
+      <c r="T30" s="13"/>
+      <c r="U30" s="29"/>
+      <c r="V30" s="31"/>
+      <c r="W30" s="29"/>
+      <c r="X30" s="25"/>
     </row>
     <row r="31" ht="12.75" customHeight="1">
-      <c r="A31" s="24"/>
-      <c r="B31" s="25"/>
-      <c r="C31" s="25"/>
-      <c r="D31" s="25"/>
-      <c r="E31" s="25"/>
-      <c r="F31" s="25"/>
-      <c r="G31" s="25"/>
-      <c r="I31" s="25"/>
-      <c r="K31" s="25"/>
-      <c r="M31" s="25"/>
-      <c r="O31" s="25"/>
-      <c r="Q31" s="25"/>
-      <c r="S31" s="25"/>
-      <c r="U31" s="25"/>
-      <c r="V31" s="26"/>
-      <c r="W31" s="25"/>
-      <c r="X31" s="27"/>
+      <c r="A31" s="21"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="29"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="29"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="30"/>
+      <c r="H31" s="13"/>
+      <c r="I31" s="30"/>
+      <c r="J31" s="13"/>
+      <c r="K31" s="30"/>
+      <c r="L31" s="13"/>
+      <c r="M31" s="30"/>
+      <c r="N31" s="13"/>
+      <c r="O31" s="30"/>
+      <c r="P31" s="13"/>
+      <c r="Q31" s="30"/>
+      <c r="R31" s="13"/>
+      <c r="S31" s="30"/>
+      <c r="T31" s="13"/>
+      <c r="U31" s="29"/>
+      <c r="V31" s="31"/>
+      <c r="W31" s="29"/>
+      <c r="X31" s="25"/>
     </row>
     <row r="32" ht="12.75" customHeight="1">
-      <c r="A32" s="24"/>
-      <c r="B32" s="25"/>
-      <c r="C32" s="25"/>
-      <c r="D32" s="25"/>
-      <c r="E32" s="25"/>
-      <c r="F32" s="25"/>
-      <c r="G32" s="25"/>
-      <c r="I32" s="25"/>
-      <c r="K32" s="25"/>
-      <c r="M32" s="25"/>
-      <c r="O32" s="25"/>
-      <c r="Q32" s="25"/>
-      <c r="S32" s="25"/>
-      <c r="U32" s="25"/>
-      <c r="V32" s="26"/>
-      <c r="W32" s="25"/>
-      <c r="X32" s="27"/>
+      <c r="A32" s="17"/>
+      <c r="B32" s="29"/>
+      <c r="C32" s="29"/>
+      <c r="D32" s="29"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="30"/>
+      <c r="H32" s="13"/>
+      <c r="I32" s="30"/>
+      <c r="J32" s="13"/>
+      <c r="K32" s="30"/>
+      <c r="L32" s="13"/>
+      <c r="M32" s="30"/>
+      <c r="N32" s="13"/>
+      <c r="O32" s="30"/>
+      <c r="P32" s="13"/>
+      <c r="Q32" s="30"/>
+      <c r="R32" s="13"/>
+      <c r="S32" s="30"/>
+      <c r="T32" s="13"/>
+      <c r="U32" s="29"/>
+      <c r="V32" s="31"/>
+      <c r="W32" s="29"/>
+      <c r="X32" s="25"/>
     </row>
     <row r="33" ht="12.75" customHeight="1">
-      <c r="A33" s="28"/>
-      <c r="B33" s="25"/>
-      <c r="C33" s="25"/>
-      <c r="D33" s="25"/>
-      <c r="E33" s="25"/>
-      <c r="F33" s="25"/>
-      <c r="G33" s="25"/>
-      <c r="I33" s="25"/>
-      <c r="K33" s="25"/>
-      <c r="M33" s="25"/>
-      <c r="O33" s="25"/>
-      <c r="Q33" s="25"/>
-      <c r="S33" s="25"/>
-      <c r="U33" s="25"/>
-      <c r="V33" s="26"/>
-      <c r="W33" s="25"/>
-      <c r="X33" s="27"/>
+      <c r="A33" s="21"/>
+      <c r="B33" s="29"/>
+      <c r="C33" s="29"/>
+      <c r="D33" s="29"/>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="30"/>
+      <c r="H33" s="13"/>
+      <c r="I33" s="30"/>
+      <c r="J33" s="13"/>
+      <c r="K33" s="30"/>
+      <c r="L33" s="13"/>
+      <c r="M33" s="30"/>
+      <c r="N33" s="13"/>
+      <c r="O33" s="30"/>
+      <c r="P33" s="13"/>
+      <c r="Q33" s="30"/>
+      <c r="R33" s="13"/>
+      <c r="S33" s="30"/>
+      <c r="T33" s="13"/>
+      <c r="U33" s="29"/>
+      <c r="V33" s="31"/>
+      <c r="W33" s="29"/>
+      <c r="X33" s="25"/>
     </row>
     <row r="34" ht="12.75" customHeight="1">
-      <c r="A34" s="24"/>
-      <c r="B34" s="25"/>
-      <c r="C34" s="25"/>
-      <c r="D34" s="25"/>
-      <c r="E34" s="25"/>
-      <c r="F34" s="25"/>
-      <c r="G34" s="25"/>
-      <c r="I34" s="25"/>
-      <c r="K34" s="25"/>
-      <c r="M34" s="25"/>
-      <c r="O34" s="25"/>
-      <c r="Q34" s="25"/>
-      <c r="S34" s="25"/>
-      <c r="U34" s="25"/>
-      <c r="V34" s="26"/>
-      <c r="W34" s="25"/>
-      <c r="X34" s="27"/>
+      <c r="A34" s="21"/>
+      <c r="B34" s="29"/>
+      <c r="C34" s="29"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="29"/>
+      <c r="G34" s="30"/>
+      <c r="H34" s="13"/>
+      <c r="I34" s="30"/>
+      <c r="J34" s="13"/>
+      <c r="K34" s="30"/>
+      <c r="L34" s="13"/>
+      <c r="M34" s="30"/>
+      <c r="N34" s="13"/>
+      <c r="O34" s="30"/>
+      <c r="P34" s="13"/>
+      <c r="Q34" s="30"/>
+      <c r="R34" s="13"/>
+      <c r="S34" s="30"/>
+      <c r="T34" s="13"/>
+      <c r="U34" s="29"/>
+      <c r="V34" s="31"/>
+      <c r="W34" s="29"/>
+      <c r="X34" s="25"/>
     </row>
     <row r="35" ht="12.75" customHeight="1">
-      <c r="A35" s="24"/>
-      <c r="B35" s="25"/>
-      <c r="C35" s="25"/>
-      <c r="D35" s="25"/>
-      <c r="E35" s="25"/>
-      <c r="F35" s="25"/>
-      <c r="G35" s="25"/>
-      <c r="I35" s="25"/>
-      <c r="K35" s="25"/>
-      <c r="M35" s="25"/>
-      <c r="O35" s="25"/>
-      <c r="Q35" s="25"/>
-      <c r="S35" s="25"/>
-      <c r="U35" s="25"/>
-      <c r="V35" s="26"/>
-      <c r="W35" s="25"/>
-      <c r="X35" s="27"/>
+      <c r="A35" s="21"/>
+      <c r="B35" s="29"/>
+      <c r="C35" s="32"/>
+      <c r="D35" s="29"/>
+      <c r="E35" s="33"/>
+      <c r="F35" s="33"/>
+      <c r="G35" s="30"/>
+      <c r="H35" s="13"/>
+      <c r="I35" s="30"/>
+      <c r="J35" s="13"/>
+      <c r="K35" s="30"/>
+      <c r="L35" s="13"/>
+      <c r="M35" s="30"/>
+      <c r="N35" s="13"/>
+      <c r="O35" s="30"/>
+      <c r="P35" s="13"/>
+      <c r="Q35" s="30"/>
+      <c r="R35" s="13"/>
+      <c r="S35" s="30"/>
+      <c r="T35" s="13"/>
+      <c r="U35" s="34"/>
+      <c r="V35" s="31"/>
+      <c r="W35" s="34"/>
+      <c r="X35" s="25"/>
     </row>
     <row r="36" ht="12.75" customHeight="1">
-      <c r="A36" s="24"/>
-      <c r="B36" s="25"/>
-      <c r="C36" s="29"/>
-      <c r="D36" s="25"/>
-      <c r="E36" s="30"/>
-      <c r="F36" s="30"/>
-      <c r="G36" s="25"/>
-      <c r="I36" s="25"/>
-      <c r="K36" s="25"/>
-      <c r="M36" s="25"/>
-      <c r="O36" s="25"/>
-      <c r="Q36" s="25"/>
-      <c r="S36" s="25"/>
-      <c r="U36" s="31"/>
-      <c r="V36" s="26"/>
-      <c r="W36" s="31"/>
-      <c r="X36" s="27"/>
+      <c r="A36" s="35"/>
+      <c r="B36" s="35"/>
+      <c r="C36" s="35"/>
+      <c r="D36" s="35"/>
+      <c r="E36" s="36"/>
+      <c r="F36" s="36"/>
+      <c r="G36" s="35"/>
+      <c r="H36" s="35"/>
+      <c r="I36" s="35"/>
+      <c r="J36" s="35"/>
+      <c r="K36" s="35"/>
+      <c r="L36" s="35"/>
+      <c r="M36" s="35"/>
+      <c r="N36" s="35"/>
+      <c r="O36" s="35"/>
+      <c r="P36" s="35"/>
+      <c r="Q36" s="35"/>
+      <c r="R36" s="35"/>
+      <c r="S36" s="35"/>
+      <c r="T36" s="35"/>
+      <c r="U36" s="35"/>
+      <c r="V36" s="35"/>
+      <c r="W36" s="35"/>
+      <c r="X36" s="25"/>
     </row>
     <row r="37" ht="12.75" customHeight="1">
-      <c r="A37" s="27"/>
-      <c r="B37" s="27"/>
-      <c r="C37" s="27"/>
-      <c r="D37" s="27"/>
-      <c r="E37" s="32"/>
-      <c r="F37" s="32"/>
-      <c r="G37" s="27"/>
-      <c r="H37" s="27"/>
-      <c r="I37" s="27"/>
-      <c r="J37" s="27"/>
-      <c r="K37" s="27"/>
-      <c r="L37" s="27"/>
-      <c r="M37" s="27"/>
-      <c r="N37" s="27"/>
-      <c r="O37" s="27"/>
-      <c r="P37" s="27"/>
-      <c r="Q37" s="27"/>
-      <c r="R37" s="27"/>
-      <c r="S37" s="27"/>
-      <c r="T37" s="27"/>
-      <c r="U37" s="27"/>
-      <c r="V37" s="27"/>
-      <c r="W37" s="27"/>
-      <c r="X37" s="27"/>
+      <c r="A37" s="35"/>
+      <c r="B37" s="35"/>
+      <c r="C37" s="35"/>
+      <c r="D37" s="35"/>
+      <c r="E37" s="36"/>
+      <c r="F37" s="36"/>
+      <c r="G37" s="35"/>
+      <c r="H37" s="35"/>
+      <c r="I37" s="35"/>
+      <c r="J37" s="35"/>
+      <c r="K37" s="35"/>
+      <c r="L37" s="35"/>
+      <c r="M37" s="35"/>
+      <c r="N37" s="35"/>
+      <c r="O37" s="35"/>
+      <c r="P37" s="35"/>
+      <c r="Q37" s="35"/>
+      <c r="R37" s="35"/>
+      <c r="S37" s="35"/>
+      <c r="T37" s="35"/>
+      <c r="U37" s="35"/>
+      <c r="V37" s="35"/>
+      <c r="W37" s="35"/>
+      <c r="X37" s="25"/>
     </row>
     <row r="38" ht="12.75" customHeight="1">
-      <c r="A38" s="27"/>
-      <c r="B38" s="27"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="27"/>
-      <c r="E38" s="32"/>
-      <c r="F38" s="32"/>
-      <c r="G38" s="27"/>
-      <c r="H38" s="27"/>
-      <c r="I38" s="27"/>
-      <c r="J38" s="27"/>
-      <c r="K38" s="27"/>
-      <c r="L38" s="27"/>
-      <c r="M38" s="27"/>
-      <c r="N38" s="27"/>
-      <c r="O38" s="27"/>
-      <c r="P38" s="27"/>
-      <c r="Q38" s="27"/>
-      <c r="R38" s="27"/>
-      <c r="S38" s="27"/>
-      <c r="T38" s="27"/>
-      <c r="U38" s="27"/>
-      <c r="V38" s="27"/>
-      <c r="W38" s="27"/>
-      <c r="X38" s="27"/>
+      <c r="A38" s="35"/>
+      <c r="B38" s="35"/>
+      <c r="C38" s="35"/>
+      <c r="D38" s="35"/>
+      <c r="E38" s="36"/>
+      <c r="F38" s="36"/>
+      <c r="G38" s="35"/>
+      <c r="H38" s="35"/>
+      <c r="I38" s="35"/>
+      <c r="J38" s="35"/>
+      <c r="K38" s="35"/>
+      <c r="L38" s="35"/>
+      <c r="M38" s="35"/>
+      <c r="N38" s="35"/>
+      <c r="O38" s="35"/>
+      <c r="P38" s="35"/>
+      <c r="Q38" s="35"/>
+      <c r="R38" s="35"/>
+      <c r="S38" s="35"/>
+      <c r="T38" s="35"/>
+      <c r="U38" s="35"/>
+      <c r="V38" s="35"/>
+      <c r="W38" s="35"/>
+      <c r="X38" s="37"/>
     </row>
     <row r="39" ht="12.75" customHeight="1">
-      <c r="A39" s="33"/>
-      <c r="B39" s="33"/>
-      <c r="C39" s="33"/>
-      <c r="D39" s="33"/>
-      <c r="E39" s="34"/>
-      <c r="F39" s="34"/>
-      <c r="G39" s="33"/>
-      <c r="H39" s="33"/>
-      <c r="I39" s="33"/>
-      <c r="J39" s="33"/>
-      <c r="K39" s="33"/>
-      <c r="L39" s="33"/>
-      <c r="M39" s="33"/>
-      <c r="N39" s="33"/>
-      <c r="O39" s="33"/>
-      <c r="P39" s="33"/>
-      <c r="Q39" s="33"/>
-      <c r="R39" s="33"/>
-      <c r="S39" s="33"/>
-      <c r="T39" s="33"/>
-      <c r="U39" s="33"/>
-      <c r="V39" s="33"/>
-      <c r="W39" s="33"/>
-      <c r="X39" s="33"/>
+      <c r="A39" s="35"/>
+      <c r="B39" s="35"/>
+      <c r="C39" s="35"/>
+      <c r="D39" s="35"/>
+      <c r="E39" s="36"/>
+      <c r="F39" s="36"/>
+      <c r="G39" s="35"/>
+      <c r="H39" s="35"/>
+      <c r="I39" s="35"/>
+      <c r="J39" s="35"/>
+      <c r="K39" s="35"/>
+      <c r="L39" s="35"/>
+      <c r="M39" s="35"/>
+      <c r="N39" s="35"/>
+      <c r="O39" s="35"/>
+      <c r="P39" s="35"/>
+      <c r="Q39" s="35"/>
+      <c r="R39" s="35"/>
+      <c r="S39" s="35"/>
+      <c r="T39" s="35"/>
+      <c r="U39" s="35"/>
+      <c r="V39" s="35"/>
+      <c r="W39" s="35"/>
+      <c r="X39" s="16"/>
     </row>
     <row r="40" ht="12.75" customHeight="1">
-      <c r="A40" s="1"/>
-      <c r="B40" s="1"/>
-      <c r="C40" s="1"/>
-      <c r="D40" s="1"/>
-      <c r="E40" s="35"/>
-      <c r="F40" s="35"/>
-      <c r="G40" s="1"/>
-      <c r="H40" s="1"/>
-      <c r="I40" s="1"/>
-      <c r="J40" s="1"/>
-      <c r="K40" s="1"/>
-      <c r="L40" s="1"/>
-      <c r="M40" s="1"/>
-      <c r="N40" s="1"/>
-      <c r="O40" s="1"/>
-      <c r="P40" s="1"/>
-      <c r="Q40" s="1"/>
-      <c r="R40" s="1"/>
-      <c r="S40" s="1"/>
-      <c r="T40" s="1"/>
-      <c r="U40" s="1"/>
-      <c r="V40" s="1"/>
-      <c r="W40" s="1"/>
-      <c r="X40" s="1"/>
+      <c r="A40" s="35"/>
+      <c r="B40" s="35"/>
+      <c r="C40" s="35"/>
+      <c r="D40" s="35"/>
+      <c r="E40" s="36"/>
+      <c r="F40" s="36"/>
+      <c r="G40" s="35"/>
+      <c r="H40" s="35"/>
+      <c r="I40" s="35"/>
+      <c r="J40" s="35"/>
+      <c r="K40" s="35"/>
+      <c r="L40" s="35"/>
+      <c r="M40" s="35"/>
+      <c r="N40" s="35"/>
+      <c r="O40" s="35"/>
+      <c r="P40" s="35"/>
+      <c r="Q40" s="35"/>
+      <c r="R40" s="35"/>
+      <c r="S40" s="35"/>
+      <c r="T40" s="35"/>
+      <c r="U40" s="35"/>
+      <c r="V40" s="35"/>
+      <c r="W40" s="35"/>
+      <c r="X40" s="16"/>
     </row>
     <row r="41" ht="12.75" customHeight="1">
-      <c r="A41" s="1"/>
-      <c r="B41" s="1"/>
-      <c r="C41" s="1"/>
-      <c r="D41" s="1"/>
-      <c r="E41" s="35"/>
-      <c r="F41" s="35"/>
-      <c r="G41" s="1"/>
-      <c r="H41" s="1"/>
-      <c r="I41" s="1"/>
-      <c r="J41" s="1"/>
-      <c r="K41" s="1"/>
-      <c r="L41" s="1"/>
-      <c r="M41" s="1"/>
-      <c r="N41" s="1"/>
-      <c r="O41" s="1"/>
-      <c r="P41" s="1"/>
-      <c r="Q41" s="1"/>
-      <c r="R41" s="1"/>
-      <c r="S41" s="1"/>
-      <c r="T41" s="1"/>
-      <c r="U41" s="1"/>
-      <c r="V41" s="1"/>
-      <c r="W41" s="1"/>
-      <c r="X41" s="1"/>
+      <c r="A41" s="35"/>
+      <c r="B41" s="35"/>
+      <c r="C41" s="35"/>
+      <c r="D41" s="35"/>
+      <c r="E41" s="36"/>
+      <c r="F41" s="36"/>
+      <c r="G41" s="35"/>
+      <c r="H41" s="35"/>
+      <c r="I41" s="35"/>
+      <c r="J41" s="35"/>
+      <c r="K41" s="35"/>
+      <c r="L41" s="35"/>
+      <c r="M41" s="35"/>
+      <c r="N41" s="35"/>
+      <c r="O41" s="35"/>
+      <c r="P41" s="35"/>
+      <c r="Q41" s="35"/>
+      <c r="R41" s="35"/>
+      <c r="S41" s="35"/>
+      <c r="T41" s="35"/>
+      <c r="U41" s="35"/>
+      <c r="V41" s="35"/>
+      <c r="W41" s="35"/>
+      <c r="X41" s="16"/>
     </row>
     <row r="42" ht="12.75" customHeight="1">
-      <c r="A42" s="1"/>
-      <c r="B42" s="1"/>
-      <c r="C42" s="1"/>
-      <c r="D42" s="1"/>
-      <c r="E42" s="35"/>
-      <c r="F42" s="35"/>
-      <c r="G42" s="1"/>
-      <c r="H42" s="1"/>
-      <c r="I42" s="1"/>
-      <c r="J42" s="1"/>
-      <c r="K42" s="1"/>
-      <c r="L42" s="1"/>
-      <c r="M42" s="1"/>
-      <c r="N42" s="1"/>
-      <c r="O42" s="1"/>
-      <c r="P42" s="1"/>
-      <c r="Q42" s="1"/>
-      <c r="R42" s="1"/>
-      <c r="S42" s="1"/>
-      <c r="T42" s="1"/>
-      <c r="U42" s="1"/>
-      <c r="V42" s="1"/>
-      <c r="W42" s="1"/>
+      <c r="A42" s="38"/>
+      <c r="B42" s="38"/>
+      <c r="C42" s="38"/>
+      <c r="D42" s="38"/>
+      <c r="E42" s="39"/>
+      <c r="F42" s="39"/>
+      <c r="G42" s="38"/>
+      <c r="H42" s="38"/>
+      <c r="I42" s="38"/>
+      <c r="J42" s="38"/>
+      <c r="K42" s="38"/>
+      <c r="L42" s="38"/>
+      <c r="M42" s="38"/>
+      <c r="N42" s="38"/>
+      <c r="O42" s="38"/>
+      <c r="P42" s="38"/>
+      <c r="Q42" s="38"/>
+      <c r="R42" s="38"/>
+      <c r="S42" s="38"/>
+      <c r="T42" s="38"/>
+      <c r="U42" s="38"/>
+      <c r="V42" s="38"/>
+      <c r="W42" s="38"/>
       <c r="X42" s="1"/>
     </row>
     <row r="43" ht="12.75" customHeight="1">
@@ -2156,8 +2480,8 @@
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
       <c r="D43" s="1"/>
-      <c r="E43" s="35"/>
-      <c r="F43" s="35"/>
+      <c r="E43" s="40"/>
+      <c r="F43" s="40"/>
       <c r="G43" s="1"/>
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
@@ -2182,8 +2506,8 @@
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
       <c r="D44" s="1"/>
-      <c r="E44" s="35"/>
-      <c r="F44" s="35"/>
+      <c r="E44" s="40"/>
+      <c r="F44" s="40"/>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
       <c r="I44" s="1"/>
@@ -2208,8 +2532,8 @@
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
       <c r="D45" s="1"/>
-      <c r="E45" s="35"/>
-      <c r="F45" s="35"/>
+      <c r="E45" s="40"/>
+      <c r="F45" s="40"/>
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
@@ -2234,8 +2558,8 @@
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
       <c r="D46" s="1"/>
-      <c r="E46" s="35"/>
-      <c r="F46" s="35"/>
+      <c r="E46" s="40"/>
+      <c r="F46" s="40"/>
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
       <c r="I46" s="1"/>
@@ -2260,8 +2584,8 @@
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
       <c r="D47" s="1"/>
-      <c r="E47" s="35"/>
-      <c r="F47" s="35"/>
+      <c r="E47" s="40"/>
+      <c r="F47" s="40"/>
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
@@ -2286,8 +2610,8 @@
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
       <c r="D48" s="1"/>
-      <c r="E48" s="35"/>
-      <c r="F48" s="35"/>
+      <c r="E48" s="40"/>
+      <c r="F48" s="40"/>
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
       <c r="I48" s="1"/>
@@ -2312,8 +2636,8 @@
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
       <c r="D49" s="1"/>
-      <c r="E49" s="35"/>
-      <c r="F49" s="35"/>
+      <c r="E49" s="40"/>
+      <c r="F49" s="40"/>
       <c r="G49" s="1"/>
       <c r="H49" s="1"/>
       <c r="I49" s="1"/>
@@ -2338,8 +2662,8 @@
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
       <c r="D50" s="1"/>
-      <c r="E50" s="35"/>
-      <c r="F50" s="35"/>
+      <c r="E50" s="40"/>
+      <c r="F50" s="40"/>
       <c r="G50" s="1"/>
       <c r="H50" s="1"/>
       <c r="I50" s="1"/>
@@ -2364,8 +2688,8 @@
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
       <c r="D51" s="1"/>
-      <c r="E51" s="35"/>
-      <c r="F51" s="35"/>
+      <c r="E51" s="40"/>
+      <c r="F51" s="40"/>
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
       <c r="I51" s="1"/>
@@ -2390,8 +2714,8 @@
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
       <c r="D52" s="1"/>
-      <c r="E52" s="35"/>
-      <c r="F52" s="35"/>
+      <c r="E52" s="40"/>
+      <c r="F52" s="40"/>
       <c r="G52" s="1"/>
       <c r="H52" s="1"/>
       <c r="I52" s="1"/>
@@ -2416,8 +2740,8 @@
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
       <c r="D53" s="1"/>
-      <c r="E53" s="35"/>
-      <c r="F53" s="35"/>
+      <c r="E53" s="40"/>
+      <c r="F53" s="40"/>
       <c r="G53" s="1"/>
       <c r="H53" s="1"/>
       <c r="I53" s="1"/>
@@ -2442,8 +2766,8 @@
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
       <c r="D54" s="1"/>
-      <c r="E54" s="35"/>
-      <c r="F54" s="35"/>
+      <c r="E54" s="40"/>
+      <c r="F54" s="40"/>
       <c r="G54" s="1"/>
       <c r="H54" s="1"/>
       <c r="I54" s="1"/>
@@ -2468,8 +2792,8 @@
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
       <c r="D55" s="1"/>
-      <c r="E55" s="35"/>
-      <c r="F55" s="35"/>
+      <c r="E55" s="40"/>
+      <c r="F55" s="40"/>
       <c r="G55" s="1"/>
       <c r="H55" s="1"/>
       <c r="I55" s="1"/>
@@ -2494,8 +2818,8 @@
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
       <c r="D56" s="1"/>
-      <c r="E56" s="35"/>
-      <c r="F56" s="35"/>
+      <c r="E56" s="40"/>
+      <c r="F56" s="40"/>
       <c r="G56" s="1"/>
       <c r="H56" s="1"/>
       <c r="I56" s="1"/>
@@ -2520,8 +2844,8 @@
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
       <c r="D57" s="1"/>
-      <c r="E57" s="35"/>
-      <c r="F57" s="35"/>
+      <c r="E57" s="40"/>
+      <c r="F57" s="40"/>
       <c r="G57" s="1"/>
       <c r="H57" s="1"/>
       <c r="I57" s="1"/>
@@ -2546,8 +2870,8 @@
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
       <c r="D58" s="1"/>
-      <c r="E58" s="35"/>
-      <c r="F58" s="35"/>
+      <c r="E58" s="40"/>
+      <c r="F58" s="40"/>
       <c r="G58" s="1"/>
       <c r="H58" s="1"/>
       <c r="I58" s="1"/>
@@ -2572,8 +2896,8 @@
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
       <c r="D59" s="1"/>
-      <c r="E59" s="35"/>
-      <c r="F59" s="35"/>
+      <c r="E59" s="40"/>
+      <c r="F59" s="40"/>
       <c r="G59" s="1"/>
       <c r="H59" s="1"/>
       <c r="I59" s="1"/>
@@ -2598,8 +2922,8 @@
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
       <c r="D60" s="1"/>
-      <c r="E60" s="35"/>
-      <c r="F60" s="35"/>
+      <c r="E60" s="40"/>
+      <c r="F60" s="40"/>
       <c r="G60" s="1"/>
       <c r="H60" s="1"/>
       <c r="I60" s="1"/>
@@ -2624,8 +2948,8 @@
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
-      <c r="E61" s="35"/>
-      <c r="F61" s="35"/>
+      <c r="E61" s="40"/>
+      <c r="F61" s="40"/>
       <c r="G61" s="1"/>
       <c r="H61" s="1"/>
       <c r="I61" s="1"/>
@@ -2650,8 +2974,8 @@
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
       <c r="D62" s="1"/>
-      <c r="E62" s="35"/>
-      <c r="F62" s="35"/>
+      <c r="E62" s="40"/>
+      <c r="F62" s="40"/>
       <c r="G62" s="1"/>
       <c r="H62" s="1"/>
       <c r="I62" s="1"/>
@@ -2676,8 +3000,8 @@
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
       <c r="D63" s="1"/>
-      <c r="E63" s="35"/>
-      <c r="F63" s="35"/>
+      <c r="E63" s="40"/>
+      <c r="F63" s="40"/>
       <c r="G63" s="1"/>
       <c r="H63" s="1"/>
       <c r="I63" s="1"/>
@@ -2702,8 +3026,8 @@
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
       <c r="D64" s="1"/>
-      <c r="E64" s="35"/>
-      <c r="F64" s="35"/>
+      <c r="E64" s="40"/>
+      <c r="F64" s="40"/>
       <c r="G64" s="1"/>
       <c r="H64" s="1"/>
       <c r="I64" s="1"/>
@@ -2728,8 +3052,8 @@
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
       <c r="D65" s="1"/>
-      <c r="E65" s="35"/>
-      <c r="F65" s="35"/>
+      <c r="E65" s="40"/>
+      <c r="F65" s="40"/>
       <c r="G65" s="1"/>
       <c r="H65" s="1"/>
       <c r="I65" s="1"/>
@@ -2754,8 +3078,8 @@
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>
       <c r="D66" s="1"/>
-      <c r="E66" s="35"/>
-      <c r="F66" s="35"/>
+      <c r="E66" s="40"/>
+      <c r="F66" s="40"/>
       <c r="G66" s="1"/>
       <c r="H66" s="1"/>
       <c r="I66" s="1"/>
@@ -2780,8 +3104,8 @@
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
       <c r="D67" s="1"/>
-      <c r="E67" s="35"/>
-      <c r="F67" s="35"/>
+      <c r="E67" s="40"/>
+      <c r="F67" s="40"/>
       <c r="G67" s="1"/>
       <c r="H67" s="1"/>
       <c r="I67" s="1"/>
@@ -2806,8 +3130,8 @@
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
       <c r="D68" s="1"/>
-      <c r="E68" s="35"/>
-      <c r="F68" s="35"/>
+      <c r="E68" s="40"/>
+      <c r="F68" s="40"/>
       <c r="G68" s="1"/>
       <c r="H68" s="1"/>
       <c r="I68" s="1"/>
@@ -2832,8 +3156,8 @@
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
       <c r="D69" s="1"/>
-      <c r="E69" s="35"/>
-      <c r="F69" s="35"/>
+      <c r="E69" s="40"/>
+      <c r="F69" s="40"/>
       <c r="G69" s="1"/>
       <c r="H69" s="1"/>
       <c r="I69" s="1"/>
@@ -2858,8 +3182,8 @@
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
       <c r="D70" s="1"/>
-      <c r="E70" s="35"/>
-      <c r="F70" s="35"/>
+      <c r="E70" s="40"/>
+      <c r="F70" s="40"/>
       <c r="G70" s="1"/>
       <c r="H70" s="1"/>
       <c r="I70" s="1"/>
@@ -2884,8 +3208,8 @@
       <c r="B71" s="1"/>
       <c r="C71" s="1"/>
       <c r="D71" s="1"/>
-      <c r="E71" s="35"/>
-      <c r="F71" s="35"/>
+      <c r="E71" s="40"/>
+      <c r="F71" s="40"/>
       <c r="G71" s="1"/>
       <c r="H71" s="1"/>
       <c r="I71" s="1"/>
@@ -2910,8 +3234,8 @@
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
       <c r="D72" s="1"/>
-      <c r="E72" s="35"/>
-      <c r="F72" s="35"/>
+      <c r="E72" s="40"/>
+      <c r="F72" s="40"/>
       <c r="G72" s="1"/>
       <c r="H72" s="1"/>
       <c r="I72" s="1"/>
@@ -2936,8 +3260,8 @@
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
       <c r="D73" s="1"/>
-      <c r="E73" s="35"/>
-      <c r="F73" s="35"/>
+      <c r="E73" s="40"/>
+      <c r="F73" s="40"/>
       <c r="G73" s="1"/>
       <c r="H73" s="1"/>
       <c r="I73" s="1"/>
@@ -2962,8 +3286,8 @@
       <c r="B74" s="1"/>
       <c r="C74" s="1"/>
       <c r="D74" s="1"/>
-      <c r="E74" s="35"/>
-      <c r="F74" s="35"/>
+      <c r="E74" s="40"/>
+      <c r="F74" s="40"/>
       <c r="G74" s="1"/>
       <c r="H74" s="1"/>
       <c r="I74" s="1"/>
@@ -2988,8 +3312,8 @@
       <c r="B75" s="1"/>
       <c r="C75" s="1"/>
       <c r="D75" s="1"/>
-      <c r="E75" s="35"/>
-      <c r="F75" s="35"/>
+      <c r="E75" s="40"/>
+      <c r="F75" s="40"/>
       <c r="G75" s="1"/>
       <c r="H75" s="1"/>
       <c r="I75" s="1"/>
@@ -3014,8 +3338,8 @@
       <c r="B76" s="1"/>
       <c r="C76" s="1"/>
       <c r="D76" s="1"/>
-      <c r="E76" s="35"/>
-      <c r="F76" s="35"/>
+      <c r="E76" s="40"/>
+      <c r="F76" s="40"/>
       <c r="G76" s="1"/>
       <c r="H76" s="1"/>
       <c r="I76" s="1"/>
@@ -3040,8 +3364,8 @@
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
       <c r="D77" s="1"/>
-      <c r="E77" s="35"/>
-      <c r="F77" s="35"/>
+      <c r="E77" s="40"/>
+      <c r="F77" s="40"/>
       <c r="G77" s="1"/>
       <c r="H77" s="1"/>
       <c r="I77" s="1"/>
@@ -3066,8 +3390,8 @@
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
       <c r="D78" s="1"/>
-      <c r="E78" s="35"/>
-      <c r="F78" s="35"/>
+      <c r="E78" s="40"/>
+      <c r="F78" s="40"/>
       <c r="G78" s="1"/>
       <c r="H78" s="1"/>
       <c r="I78" s="1"/>
@@ -3092,8 +3416,8 @@
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
       <c r="D79" s="1"/>
-      <c r="E79" s="35"/>
-      <c r="F79" s="35"/>
+      <c r="E79" s="40"/>
+      <c r="F79" s="40"/>
       <c r="G79" s="1"/>
       <c r="H79" s="1"/>
       <c r="I79" s="1"/>
@@ -3118,8 +3442,8 @@
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
       <c r="D80" s="1"/>
-      <c r="E80" s="35"/>
-      <c r="F80" s="35"/>
+      <c r="E80" s="40"/>
+      <c r="F80" s="40"/>
       <c r="G80" s="1"/>
       <c r="H80" s="1"/>
       <c r="I80" s="1"/>
@@ -3144,8 +3468,8 @@
       <c r="B81" s="1"/>
       <c r="C81" s="1"/>
       <c r="D81" s="1"/>
-      <c r="E81" s="35"/>
-      <c r="F81" s="35"/>
+      <c r="E81" s="40"/>
+      <c r="F81" s="40"/>
       <c r="G81" s="1"/>
       <c r="H81" s="1"/>
       <c r="I81" s="1"/>
@@ -3170,8 +3494,8 @@
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
       <c r="D82" s="1"/>
-      <c r="E82" s="35"/>
-      <c r="F82" s="35"/>
+      <c r="E82" s="40"/>
+      <c r="F82" s="40"/>
       <c r="G82" s="1"/>
       <c r="H82" s="1"/>
       <c r="I82" s="1"/>
@@ -3196,8 +3520,8 @@
       <c r="B83" s="1"/>
       <c r="C83" s="1"/>
       <c r="D83" s="1"/>
-      <c r="E83" s="35"/>
-      <c r="F83" s="35"/>
+      <c r="E83" s="40"/>
+      <c r="F83" s="40"/>
       <c r="G83" s="1"/>
       <c r="H83" s="1"/>
       <c r="I83" s="1"/>
@@ -3222,8 +3546,8 @@
       <c r="B84" s="1"/>
       <c r="C84" s="1"/>
       <c r="D84" s="1"/>
-      <c r="E84" s="35"/>
-      <c r="F84" s="35"/>
+      <c r="E84" s="40"/>
+      <c r="F84" s="40"/>
       <c r="G84" s="1"/>
       <c r="H84" s="1"/>
       <c r="I84" s="1"/>
@@ -3248,8 +3572,8 @@
       <c r="B85" s="1"/>
       <c r="C85" s="1"/>
       <c r="D85" s="1"/>
-      <c r="E85" s="35"/>
-      <c r="F85" s="35"/>
+      <c r="E85" s="40"/>
+      <c r="F85" s="40"/>
       <c r="G85" s="1"/>
       <c r="H85" s="1"/>
       <c r="I85" s="1"/>
@@ -3274,8 +3598,8 @@
       <c r="B86" s="1"/>
       <c r="C86" s="1"/>
       <c r="D86" s="1"/>
-      <c r="E86" s="35"/>
-      <c r="F86" s="35"/>
+      <c r="E86" s="40"/>
+      <c r="F86" s="40"/>
       <c r="G86" s="1"/>
       <c r="H86" s="1"/>
       <c r="I86" s="1"/>
@@ -3300,8 +3624,8 @@
       <c r="B87" s="1"/>
       <c r="C87" s="1"/>
       <c r="D87" s="1"/>
-      <c r="E87" s="35"/>
-      <c r="F87" s="35"/>
+      <c r="E87" s="40"/>
+      <c r="F87" s="40"/>
       <c r="G87" s="1"/>
       <c r="H87" s="1"/>
       <c r="I87" s="1"/>
@@ -3326,8 +3650,8 @@
       <c r="B88" s="1"/>
       <c r="C88" s="1"/>
       <c r="D88" s="1"/>
-      <c r="E88" s="35"/>
-      <c r="F88" s="35"/>
+      <c r="E88" s="40"/>
+      <c r="F88" s="40"/>
       <c r="G88" s="1"/>
       <c r="H88" s="1"/>
       <c r="I88" s="1"/>
@@ -3352,8 +3676,8 @@
       <c r="B89" s="1"/>
       <c r="C89" s="1"/>
       <c r="D89" s="1"/>
-      <c r="E89" s="35"/>
-      <c r="F89" s="35"/>
+      <c r="E89" s="40"/>
+      <c r="F89" s="40"/>
       <c r="G89" s="1"/>
       <c r="H89" s="1"/>
       <c r="I89" s="1"/>
@@ -3378,8 +3702,8 @@
       <c r="B90" s="1"/>
       <c r="C90" s="1"/>
       <c r="D90" s="1"/>
-      <c r="E90" s="35"/>
-      <c r="F90" s="35"/>
+      <c r="E90" s="40"/>
+      <c r="F90" s="40"/>
       <c r="G90" s="1"/>
       <c r="H90" s="1"/>
       <c r="I90" s="1"/>
@@ -3404,8 +3728,8 @@
       <c r="B91" s="1"/>
       <c r="C91" s="1"/>
       <c r="D91" s="1"/>
-      <c r="E91" s="35"/>
-      <c r="F91" s="35"/>
+      <c r="E91" s="40"/>
+      <c r="F91" s="40"/>
       <c r="G91" s="1"/>
       <c r="H91" s="1"/>
       <c r="I91" s="1"/>
@@ -3430,8 +3754,8 @@
       <c r="B92" s="1"/>
       <c r="C92" s="1"/>
       <c r="D92" s="1"/>
-      <c r="E92" s="35"/>
-      <c r="F92" s="35"/>
+      <c r="E92" s="40"/>
+      <c r="F92" s="40"/>
       <c r="G92" s="1"/>
       <c r="H92" s="1"/>
       <c r="I92" s="1"/>
@@ -3456,8 +3780,8 @@
       <c r="B93" s="1"/>
       <c r="C93" s="1"/>
       <c r="D93" s="1"/>
-      <c r="E93" s="35"/>
-      <c r="F93" s="35"/>
+      <c r="E93" s="40"/>
+      <c r="F93" s="40"/>
       <c r="G93" s="1"/>
       <c r="H93" s="1"/>
       <c r="I93" s="1"/>
@@ -3482,8 +3806,8 @@
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
       <c r="D94" s="1"/>
-      <c r="E94" s="35"/>
-      <c r="F94" s="35"/>
+      <c r="E94" s="40"/>
+      <c r="F94" s="40"/>
       <c r="G94" s="1"/>
       <c r="H94" s="1"/>
       <c r="I94" s="1"/>
@@ -3508,8 +3832,8 @@
       <c r="B95" s="1"/>
       <c r="C95" s="1"/>
       <c r="D95" s="1"/>
-      <c r="E95" s="35"/>
-      <c r="F95" s="35"/>
+      <c r="E95" s="40"/>
+      <c r="F95" s="40"/>
       <c r="G95" s="1"/>
       <c r="H95" s="1"/>
       <c r="I95" s="1"/>
@@ -3534,8 +3858,8 @@
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
       <c r="D96" s="1"/>
-      <c r="E96" s="35"/>
-      <c r="F96" s="35"/>
+      <c r="E96" s="40"/>
+      <c r="F96" s="40"/>
       <c r="G96" s="1"/>
       <c r="H96" s="1"/>
       <c r="I96" s="1"/>
@@ -3560,8 +3884,8 @@
       <c r="B97" s="1"/>
       <c r="C97" s="1"/>
       <c r="D97" s="1"/>
-      <c r="E97" s="35"/>
-      <c r="F97" s="35"/>
+      <c r="E97" s="40"/>
+      <c r="F97" s="40"/>
       <c r="G97" s="1"/>
       <c r="H97" s="1"/>
       <c r="I97" s="1"/>
@@ -3586,8 +3910,8 @@
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
       <c r="D98" s="1"/>
-      <c r="E98" s="35"/>
-      <c r="F98" s="35"/>
+      <c r="E98" s="40"/>
+      <c r="F98" s="40"/>
       <c r="G98" s="1"/>
       <c r="H98" s="1"/>
       <c r="I98" s="1"/>
@@ -3612,8 +3936,8 @@
       <c r="B99" s="1"/>
       <c r="C99" s="1"/>
       <c r="D99" s="1"/>
-      <c r="E99" s="35"/>
-      <c r="F99" s="35"/>
+      <c r="E99" s="40"/>
+      <c r="F99" s="40"/>
       <c r="G99" s="1"/>
       <c r="H99" s="1"/>
       <c r="I99" s="1"/>
@@ -3638,8 +3962,8 @@
       <c r="B100" s="1"/>
       <c r="C100" s="1"/>
       <c r="D100" s="1"/>
-      <c r="E100" s="35"/>
-      <c r="F100" s="35"/>
+      <c r="E100" s="40"/>
+      <c r="F100" s="40"/>
       <c r="G100" s="1"/>
       <c r="H100" s="1"/>
       <c r="I100" s="1"/>
@@ -3664,8 +3988,8 @@
       <c r="B101" s="1"/>
       <c r="C101" s="1"/>
       <c r="D101" s="1"/>
-      <c r="E101" s="35"/>
-      <c r="F101" s="35"/>
+      <c r="E101" s="40"/>
+      <c r="F101" s="40"/>
       <c r="G101" s="1"/>
       <c r="H101" s="1"/>
       <c r="I101" s="1"/>
@@ -3690,8 +4014,8 @@
       <c r="B102" s="1"/>
       <c r="C102" s="1"/>
       <c r="D102" s="1"/>
-      <c r="E102" s="35"/>
-      <c r="F102" s="35"/>
+      <c r="E102" s="40"/>
+      <c r="F102" s="40"/>
       <c r="G102" s="1"/>
       <c r="H102" s="1"/>
       <c r="I102" s="1"/>
@@ -3716,8 +4040,8 @@
       <c r="B103" s="1"/>
       <c r="C103" s="1"/>
       <c r="D103" s="1"/>
-      <c r="E103" s="35"/>
-      <c r="F103" s="35"/>
+      <c r="E103" s="40"/>
+      <c r="F103" s="40"/>
       <c r="G103" s="1"/>
       <c r="H103" s="1"/>
       <c r="I103" s="1"/>
@@ -3742,8 +4066,8 @@
       <c r="B104" s="1"/>
       <c r="C104" s="1"/>
       <c r="D104" s="1"/>
-      <c r="E104" s="35"/>
-      <c r="F104" s="35"/>
+      <c r="E104" s="40"/>
+      <c r="F104" s="40"/>
       <c r="G104" s="1"/>
       <c r="H104" s="1"/>
       <c r="I104" s="1"/>
@@ -3768,8 +4092,8 @@
       <c r="B105" s="1"/>
       <c r="C105" s="1"/>
       <c r="D105" s="1"/>
-      <c r="E105" s="35"/>
-      <c r="F105" s="35"/>
+      <c r="E105" s="40"/>
+      <c r="F105" s="40"/>
       <c r="G105" s="1"/>
       <c r="H105" s="1"/>
       <c r="I105" s="1"/>
@@ -3794,8 +4118,8 @@
       <c r="B106" s="1"/>
       <c r="C106" s="1"/>
       <c r="D106" s="1"/>
-      <c r="E106" s="35"/>
-      <c r="F106" s="35"/>
+      <c r="E106" s="40"/>
+      <c r="F106" s="40"/>
       <c r="G106" s="1"/>
       <c r="H106" s="1"/>
       <c r="I106" s="1"/>
@@ -3820,8 +4144,8 @@
       <c r="B107" s="1"/>
       <c r="C107" s="1"/>
       <c r="D107" s="1"/>
-      <c r="E107" s="35"/>
-      <c r="F107" s="35"/>
+      <c r="E107" s="40"/>
+      <c r="F107" s="40"/>
       <c r="G107" s="1"/>
       <c r="H107" s="1"/>
       <c r="I107" s="1"/>
@@ -3846,8 +4170,8 @@
       <c r="B108" s="1"/>
       <c r="C108" s="1"/>
       <c r="D108" s="1"/>
-      <c r="E108" s="35"/>
-      <c r="F108" s="35"/>
+      <c r="E108" s="40"/>
+      <c r="F108" s="40"/>
       <c r="G108" s="1"/>
       <c r="H108" s="1"/>
       <c r="I108" s="1"/>
@@ -3872,8 +4196,8 @@
       <c r="B109" s="1"/>
       <c r="C109" s="1"/>
       <c r="D109" s="1"/>
-      <c r="E109" s="35"/>
-      <c r="F109" s="35"/>
+      <c r="E109" s="40"/>
+      <c r="F109" s="40"/>
       <c r="G109" s="1"/>
       <c r="H109" s="1"/>
       <c r="I109" s="1"/>
@@ -3898,8 +4222,8 @@
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
       <c r="D110" s="1"/>
-      <c r="E110" s="35"/>
-      <c r="F110" s="35"/>
+      <c r="E110" s="40"/>
+      <c r="F110" s="40"/>
       <c r="G110" s="1"/>
       <c r="H110" s="1"/>
       <c r="I110" s="1"/>
@@ -3924,8 +4248,8 @@
       <c r="B111" s="1"/>
       <c r="C111" s="1"/>
       <c r="D111" s="1"/>
-      <c r="E111" s="35"/>
-      <c r="F111" s="35"/>
+      <c r="E111" s="40"/>
+      <c r="F111" s="40"/>
       <c r="G111" s="1"/>
       <c r="H111" s="1"/>
       <c r="I111" s="1"/>
@@ -3950,8 +4274,8 @@
       <c r="B112" s="1"/>
       <c r="C112" s="1"/>
       <c r="D112" s="1"/>
-      <c r="E112" s="35"/>
-      <c r="F112" s="35"/>
+      <c r="E112" s="40"/>
+      <c r="F112" s="40"/>
       <c r="G112" s="1"/>
       <c r="H112" s="1"/>
       <c r="I112" s="1"/>
@@ -3976,8 +4300,8 @@
       <c r="B113" s="1"/>
       <c r="C113" s="1"/>
       <c r="D113" s="1"/>
-      <c r="E113" s="35"/>
-      <c r="F113" s="35"/>
+      <c r="E113" s="40"/>
+      <c r="F113" s="40"/>
       <c r="G113" s="1"/>
       <c r="H113" s="1"/>
       <c r="I113" s="1"/>
@@ -4002,8 +4326,8 @@
       <c r="B114" s="1"/>
       <c r="C114" s="1"/>
       <c r="D114" s="1"/>
-      <c r="E114" s="35"/>
-      <c r="F114" s="35"/>
+      <c r="E114" s="40"/>
+      <c r="F114" s="40"/>
       <c r="G114" s="1"/>
       <c r="H114" s="1"/>
       <c r="I114" s="1"/>
@@ -4028,8 +4352,8 @@
       <c r="B115" s="1"/>
       <c r="C115" s="1"/>
       <c r="D115" s="1"/>
-      <c r="E115" s="35"/>
-      <c r="F115" s="35"/>
+      <c r="E115" s="40"/>
+      <c r="F115" s="40"/>
       <c r="G115" s="1"/>
       <c r="H115" s="1"/>
       <c r="I115" s="1"/>
@@ -4054,8 +4378,8 @@
       <c r="B116" s="1"/>
       <c r="C116" s="1"/>
       <c r="D116" s="1"/>
-      <c r="E116" s="35"/>
-      <c r="F116" s="35"/>
+      <c r="E116" s="40"/>
+      <c r="F116" s="40"/>
       <c r="G116" s="1"/>
       <c r="H116" s="1"/>
       <c r="I116" s="1"/>
@@ -4080,8 +4404,8 @@
       <c r="B117" s="1"/>
       <c r="C117" s="1"/>
       <c r="D117" s="1"/>
-      <c r="E117" s="35"/>
-      <c r="F117" s="35"/>
+      <c r="E117" s="40"/>
+      <c r="F117" s="40"/>
       <c r="G117" s="1"/>
       <c r="H117" s="1"/>
       <c r="I117" s="1"/>
@@ -4106,8 +4430,8 @@
       <c r="B118" s="1"/>
       <c r="C118" s="1"/>
       <c r="D118" s="1"/>
-      <c r="E118" s="35"/>
-      <c r="F118" s="35"/>
+      <c r="E118" s="40"/>
+      <c r="F118" s="40"/>
       <c r="G118" s="1"/>
       <c r="H118" s="1"/>
       <c r="I118" s="1"/>
@@ -4132,8 +4456,8 @@
       <c r="B119" s="1"/>
       <c r="C119" s="1"/>
       <c r="D119" s="1"/>
-      <c r="E119" s="35"/>
-      <c r="F119" s="35"/>
+      <c r="E119" s="40"/>
+      <c r="F119" s="40"/>
       <c r="G119" s="1"/>
       <c r="H119" s="1"/>
       <c r="I119" s="1"/>
@@ -4158,8 +4482,8 @@
       <c r="B120" s="1"/>
       <c r="C120" s="1"/>
       <c r="D120" s="1"/>
-      <c r="E120" s="35"/>
-      <c r="F120" s="35"/>
+      <c r="E120" s="40"/>
+      <c r="F120" s="40"/>
       <c r="G120" s="1"/>
       <c r="H120" s="1"/>
       <c r="I120" s="1"/>
@@ -4184,8 +4508,8 @@
       <c r="B121" s="1"/>
       <c r="C121" s="1"/>
       <c r="D121" s="1"/>
-      <c r="E121" s="35"/>
-      <c r="F121" s="35"/>
+      <c r="E121" s="40"/>
+      <c r="F121" s="40"/>
       <c r="G121" s="1"/>
       <c r="H121" s="1"/>
       <c r="I121" s="1"/>
@@ -4210,8 +4534,8 @@
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
       <c r="D122" s="1"/>
-      <c r="E122" s="35"/>
-      <c r="F122" s="35"/>
+      <c r="E122" s="40"/>
+      <c r="F122" s="40"/>
       <c r="G122" s="1"/>
       <c r="H122" s="1"/>
       <c r="I122" s="1"/>
@@ -4236,8 +4560,8 @@
       <c r="B123" s="1"/>
       <c r="C123" s="1"/>
       <c r="D123" s="1"/>
-      <c r="E123" s="35"/>
-      <c r="F123" s="35"/>
+      <c r="E123" s="40"/>
+      <c r="F123" s="40"/>
       <c r="G123" s="1"/>
       <c r="H123" s="1"/>
       <c r="I123" s="1"/>
@@ -4262,8 +4586,8 @@
       <c r="B124" s="1"/>
       <c r="C124" s="1"/>
       <c r="D124" s="1"/>
-      <c r="E124" s="35"/>
-      <c r="F124" s="35"/>
+      <c r="E124" s="40"/>
+      <c r="F124" s="40"/>
       <c r="G124" s="1"/>
       <c r="H124" s="1"/>
       <c r="I124" s="1"/>
@@ -4288,8 +4612,8 @@
       <c r="B125" s="1"/>
       <c r="C125" s="1"/>
       <c r="D125" s="1"/>
-      <c r="E125" s="35"/>
-      <c r="F125" s="35"/>
+      <c r="E125" s="40"/>
+      <c r="F125" s="40"/>
       <c r="G125" s="1"/>
       <c r="H125" s="1"/>
       <c r="I125" s="1"/>
@@ -4314,8 +4638,8 @@
       <c r="B126" s="1"/>
       <c r="C126" s="1"/>
       <c r="D126" s="1"/>
-      <c r="E126" s="35"/>
-      <c r="F126" s="35"/>
+      <c r="E126" s="40"/>
+      <c r="F126" s="40"/>
       <c r="G126" s="1"/>
       <c r="H126" s="1"/>
       <c r="I126" s="1"/>
@@ -4340,8 +4664,8 @@
       <c r="B127" s="1"/>
       <c r="C127" s="1"/>
       <c r="D127" s="1"/>
-      <c r="E127" s="35"/>
-      <c r="F127" s="35"/>
+      <c r="E127" s="40"/>
+      <c r="F127" s="40"/>
       <c r="G127" s="1"/>
       <c r="H127" s="1"/>
       <c r="I127" s="1"/>
@@ -4366,8 +4690,8 @@
       <c r="B128" s="1"/>
       <c r="C128" s="1"/>
       <c r="D128" s="1"/>
-      <c r="E128" s="35"/>
-      <c r="F128" s="35"/>
+      <c r="E128" s="40"/>
+      <c r="F128" s="40"/>
       <c r="G128" s="1"/>
       <c r="H128" s="1"/>
       <c r="I128" s="1"/>
@@ -4392,8 +4716,8 @@
       <c r="B129" s="1"/>
       <c r="C129" s="1"/>
       <c r="D129" s="1"/>
-      <c r="E129" s="35"/>
-      <c r="F129" s="35"/>
+      <c r="E129" s="40"/>
+      <c r="F129" s="40"/>
       <c r="G129" s="1"/>
       <c r="H129" s="1"/>
       <c r="I129" s="1"/>
@@ -4418,8 +4742,8 @@
       <c r="B130" s="1"/>
       <c r="C130" s="1"/>
       <c r="D130" s="1"/>
-      <c r="E130" s="35"/>
-      <c r="F130" s="35"/>
+      <c r="E130" s="40"/>
+      <c r="F130" s="40"/>
       <c r="G130" s="1"/>
       <c r="H130" s="1"/>
       <c r="I130" s="1"/>
@@ -4444,8 +4768,8 @@
       <c r="B131" s="1"/>
       <c r="C131" s="1"/>
       <c r="D131" s="1"/>
-      <c r="E131" s="35"/>
-      <c r="F131" s="35"/>
+      <c r="E131" s="40"/>
+      <c r="F131" s="40"/>
       <c r="G131" s="1"/>
       <c r="H131" s="1"/>
       <c r="I131" s="1"/>
@@ -4470,8 +4794,8 @@
       <c r="B132" s="1"/>
       <c r="C132" s="1"/>
       <c r="D132" s="1"/>
-      <c r="E132" s="35"/>
-      <c r="F132" s="35"/>
+      <c r="E132" s="40"/>
+      <c r="F132" s="40"/>
       <c r="G132" s="1"/>
       <c r="H132" s="1"/>
       <c r="I132" s="1"/>
@@ -4496,8 +4820,8 @@
       <c r="B133" s="1"/>
       <c r="C133" s="1"/>
       <c r="D133" s="1"/>
-      <c r="E133" s="35"/>
-      <c r="F133" s="35"/>
+      <c r="E133" s="40"/>
+      <c r="F133" s="40"/>
       <c r="G133" s="1"/>
       <c r="H133" s="1"/>
       <c r="I133" s="1"/>
@@ -4522,8 +4846,8 @@
       <c r="B134" s="1"/>
       <c r="C134" s="1"/>
       <c r="D134" s="1"/>
-      <c r="E134" s="35"/>
-      <c r="F134" s="35"/>
+      <c r="E134" s="40"/>
+      <c r="F134" s="40"/>
       <c r="G134" s="1"/>
       <c r="H134" s="1"/>
       <c r="I134" s="1"/>
@@ -4548,8 +4872,8 @@
       <c r="B135" s="1"/>
       <c r="C135" s="1"/>
       <c r="D135" s="1"/>
-      <c r="E135" s="35"/>
-      <c r="F135" s="35"/>
+      <c r="E135" s="40"/>
+      <c r="F135" s="40"/>
       <c r="G135" s="1"/>
       <c r="H135" s="1"/>
       <c r="I135" s="1"/>
@@ -4574,8 +4898,8 @@
       <c r="B136" s="1"/>
       <c r="C136" s="1"/>
       <c r="D136" s="1"/>
-      <c r="E136" s="35"/>
-      <c r="F136" s="35"/>
+      <c r="E136" s="40"/>
+      <c r="F136" s="40"/>
       <c r="G136" s="1"/>
       <c r="H136" s="1"/>
       <c r="I136" s="1"/>
@@ -4600,8 +4924,8 @@
       <c r="B137" s="1"/>
       <c r="C137" s="1"/>
       <c r="D137" s="1"/>
-      <c r="E137" s="35"/>
-      <c r="F137" s="35"/>
+      <c r="E137" s="40"/>
+      <c r="F137" s="40"/>
       <c r="G137" s="1"/>
       <c r="H137" s="1"/>
       <c r="I137" s="1"/>
@@ -4626,8 +4950,8 @@
       <c r="B138" s="1"/>
       <c r="C138" s="1"/>
       <c r="D138" s="1"/>
-      <c r="E138" s="35"/>
-      <c r="F138" s="35"/>
+      <c r="E138" s="40"/>
+      <c r="F138" s="40"/>
       <c r="G138" s="1"/>
       <c r="H138" s="1"/>
       <c r="I138" s="1"/>
@@ -4652,8 +4976,8 @@
       <c r="B139" s="1"/>
       <c r="C139" s="1"/>
       <c r="D139" s="1"/>
-      <c r="E139" s="35"/>
-      <c r="F139" s="35"/>
+      <c r="E139" s="40"/>
+      <c r="F139" s="40"/>
       <c r="G139" s="1"/>
       <c r="H139" s="1"/>
       <c r="I139" s="1"/>
@@ -4678,8 +5002,8 @@
       <c r="B140" s="1"/>
       <c r="C140" s="1"/>
       <c r="D140" s="1"/>
-      <c r="E140" s="35"/>
-      <c r="F140" s="35"/>
+      <c r="E140" s="40"/>
+      <c r="F140" s="40"/>
       <c r="G140" s="1"/>
       <c r="H140" s="1"/>
       <c r="I140" s="1"/>
@@ -4704,8 +5028,8 @@
       <c r="B141" s="1"/>
       <c r="C141" s="1"/>
       <c r="D141" s="1"/>
-      <c r="E141" s="35"/>
-      <c r="F141" s="35"/>
+      <c r="E141" s="40"/>
+      <c r="F141" s="40"/>
       <c r="G141" s="1"/>
       <c r="H141" s="1"/>
       <c r="I141" s="1"/>
@@ -4730,8 +5054,8 @@
       <c r="B142" s="1"/>
       <c r="C142" s="1"/>
       <c r="D142" s="1"/>
-      <c r="E142" s="35"/>
-      <c r="F142" s="35"/>
+      <c r="E142" s="40"/>
+      <c r="F142" s="40"/>
       <c r="G142" s="1"/>
       <c r="H142" s="1"/>
       <c r="I142" s="1"/>
@@ -4756,8 +5080,8 @@
       <c r="B143" s="1"/>
       <c r="C143" s="1"/>
       <c r="D143" s="1"/>
-      <c r="E143" s="35"/>
-      <c r="F143" s="35"/>
+      <c r="E143" s="40"/>
+      <c r="F143" s="40"/>
       <c r="G143" s="1"/>
       <c r="H143" s="1"/>
       <c r="I143" s="1"/>
@@ -4782,8 +5106,8 @@
       <c r="B144" s="1"/>
       <c r="C144" s="1"/>
       <c r="D144" s="1"/>
-      <c r="E144" s="35"/>
-      <c r="F144" s="35"/>
+      <c r="E144" s="40"/>
+      <c r="F144" s="40"/>
       <c r="G144" s="1"/>
       <c r="H144" s="1"/>
       <c r="I144" s="1"/>
@@ -4808,8 +5132,8 @@
       <c r="B145" s="1"/>
       <c r="C145" s="1"/>
       <c r="D145" s="1"/>
-      <c r="E145" s="35"/>
-      <c r="F145" s="35"/>
+      <c r="E145" s="40"/>
+      <c r="F145" s="40"/>
       <c r="G145" s="1"/>
       <c r="H145" s="1"/>
       <c r="I145" s="1"/>
@@ -4834,8 +5158,8 @@
       <c r="B146" s="1"/>
       <c r="C146" s="1"/>
       <c r="D146" s="1"/>
-      <c r="E146" s="35"/>
-      <c r="F146" s="35"/>
+      <c r="E146" s="40"/>
+      <c r="F146" s="40"/>
       <c r="G146" s="1"/>
       <c r="H146" s="1"/>
       <c r="I146" s="1"/>
@@ -4860,8 +5184,8 @@
       <c r="B147" s="1"/>
       <c r="C147" s="1"/>
       <c r="D147" s="1"/>
-      <c r="E147" s="35"/>
-      <c r="F147" s="35"/>
+      <c r="E147" s="40"/>
+      <c r="F147" s="40"/>
       <c r="G147" s="1"/>
       <c r="H147" s="1"/>
       <c r="I147" s="1"/>
@@ -4886,8 +5210,8 @@
       <c r="B148" s="1"/>
       <c r="C148" s="1"/>
       <c r="D148" s="1"/>
-      <c r="E148" s="35"/>
-      <c r="F148" s="35"/>
+      <c r="E148" s="40"/>
+      <c r="F148" s="40"/>
       <c r="G148" s="1"/>
       <c r="H148" s="1"/>
       <c r="I148" s="1"/>
@@ -4912,8 +5236,8 @@
       <c r="B149" s="1"/>
       <c r="C149" s="1"/>
       <c r="D149" s="1"/>
-      <c r="E149" s="35"/>
-      <c r="F149" s="35"/>
+      <c r="E149" s="40"/>
+      <c r="F149" s="40"/>
       <c r="G149" s="1"/>
       <c r="H149" s="1"/>
       <c r="I149" s="1"/>
@@ -4938,8 +5262,8 @@
       <c r="B150" s="1"/>
       <c r="C150" s="1"/>
       <c r="D150" s="1"/>
-      <c r="E150" s="35"/>
-      <c r="F150" s="35"/>
+      <c r="E150" s="40"/>
+      <c r="F150" s="40"/>
       <c r="G150" s="1"/>
       <c r="H150" s="1"/>
       <c r="I150" s="1"/>
@@ -4964,8 +5288,8 @@
       <c r="B151" s="1"/>
       <c r="C151" s="1"/>
       <c r="D151" s="1"/>
-      <c r="E151" s="35"/>
-      <c r="F151" s="35"/>
+      <c r="E151" s="40"/>
+      <c r="F151" s="40"/>
       <c r="G151" s="1"/>
       <c r="H151" s="1"/>
       <c r="I151" s="1"/>
@@ -4990,8 +5314,8 @@
       <c r="B152" s="1"/>
       <c r="C152" s="1"/>
       <c r="D152" s="1"/>
-      <c r="E152" s="35"/>
-      <c r="F152" s="35"/>
+      <c r="E152" s="40"/>
+      <c r="F152" s="40"/>
       <c r="G152" s="1"/>
       <c r="H152" s="1"/>
       <c r="I152" s="1"/>
@@ -5016,8 +5340,8 @@
       <c r="B153" s="1"/>
       <c r="C153" s="1"/>
       <c r="D153" s="1"/>
-      <c r="E153" s="35"/>
-      <c r="F153" s="35"/>
+      <c r="E153" s="40"/>
+      <c r="F153" s="40"/>
       <c r="G153" s="1"/>
       <c r="H153" s="1"/>
       <c r="I153" s="1"/>
@@ -5042,8 +5366,8 @@
       <c r="B154" s="1"/>
       <c r="C154" s="1"/>
       <c r="D154" s="1"/>
-      <c r="E154" s="35"/>
-      <c r="F154" s="35"/>
+      <c r="E154" s="40"/>
+      <c r="F154" s="40"/>
       <c r="G154" s="1"/>
       <c r="H154" s="1"/>
       <c r="I154" s="1"/>
@@ -5068,8 +5392,8 @@
       <c r="B155" s="1"/>
       <c r="C155" s="1"/>
       <c r="D155" s="1"/>
-      <c r="E155" s="35"/>
-      <c r="F155" s="35"/>
+      <c r="E155" s="40"/>
+      <c r="F155" s="40"/>
       <c r="G155" s="1"/>
       <c r="H155" s="1"/>
       <c r="I155" s="1"/>
@@ -5094,8 +5418,8 @@
       <c r="B156" s="1"/>
       <c r="C156" s="1"/>
       <c r="D156" s="1"/>
-      <c r="E156" s="35"/>
-      <c r="F156" s="35"/>
+      <c r="E156" s="40"/>
+      <c r="F156" s="40"/>
       <c r="G156" s="1"/>
       <c r="H156" s="1"/>
       <c r="I156" s="1"/>
@@ -5120,8 +5444,8 @@
       <c r="B157" s="1"/>
       <c r="C157" s="1"/>
       <c r="D157" s="1"/>
-      <c r="E157" s="35"/>
-      <c r="F157" s="35"/>
+      <c r="E157" s="40"/>
+      <c r="F157" s="40"/>
       <c r="G157" s="1"/>
       <c r="H157" s="1"/>
       <c r="I157" s="1"/>
@@ -5146,8 +5470,8 @@
       <c r="B158" s="1"/>
       <c r="C158" s="1"/>
       <c r="D158" s="1"/>
-      <c r="E158" s="35"/>
-      <c r="F158" s="35"/>
+      <c r="E158" s="40"/>
+      <c r="F158" s="40"/>
       <c r="G158" s="1"/>
       <c r="H158" s="1"/>
       <c r="I158" s="1"/>
@@ -5172,8 +5496,8 @@
       <c r="B159" s="1"/>
       <c r="C159" s="1"/>
       <c r="D159" s="1"/>
-      <c r="E159" s="35"/>
-      <c r="F159" s="35"/>
+      <c r="E159" s="40"/>
+      <c r="F159" s="40"/>
       <c r="G159" s="1"/>
       <c r="H159" s="1"/>
       <c r="I159" s="1"/>
@@ -5198,8 +5522,8 @@
       <c r="B160" s="1"/>
       <c r="C160" s="1"/>
       <c r="D160" s="1"/>
-      <c r="E160" s="35"/>
-      <c r="F160" s="35"/>
+      <c r="E160" s="40"/>
+      <c r="F160" s="40"/>
       <c r="G160" s="1"/>
       <c r="H160" s="1"/>
       <c r="I160" s="1"/>
@@ -5224,8 +5548,8 @@
       <c r="B161" s="1"/>
       <c r="C161" s="1"/>
       <c r="D161" s="1"/>
-      <c r="E161" s="35"/>
-      <c r="F161" s="35"/>
+      <c r="E161" s="40"/>
+      <c r="F161" s="40"/>
       <c r="G161" s="1"/>
       <c r="H161" s="1"/>
       <c r="I161" s="1"/>
@@ -5250,8 +5574,8 @@
       <c r="B162" s="1"/>
       <c r="C162" s="1"/>
       <c r="D162" s="1"/>
-      <c r="E162" s="35"/>
-      <c r="F162" s="35"/>
+      <c r="E162" s="40"/>
+      <c r="F162" s="40"/>
       <c r="G162" s="1"/>
       <c r="H162" s="1"/>
       <c r="I162" s="1"/>
@@ -5276,8 +5600,8 @@
       <c r="B163" s="1"/>
       <c r="C163" s="1"/>
       <c r="D163" s="1"/>
-      <c r="E163" s="35"/>
-      <c r="F163" s="35"/>
+      <c r="E163" s="40"/>
+      <c r="F163" s="40"/>
       <c r="G163" s="1"/>
       <c r="H163" s="1"/>
       <c r="I163" s="1"/>
@@ -5302,8 +5626,8 @@
       <c r="B164" s="1"/>
       <c r="C164" s="1"/>
       <c r="D164" s="1"/>
-      <c r="E164" s="35"/>
-      <c r="F164" s="35"/>
+      <c r="E164" s="40"/>
+      <c r="F164" s="40"/>
       <c r="G164" s="1"/>
       <c r="H164" s="1"/>
       <c r="I164" s="1"/>
@@ -5328,8 +5652,8 @@
       <c r="B165" s="1"/>
       <c r="C165" s="1"/>
       <c r="D165" s="1"/>
-      <c r="E165" s="35"/>
-      <c r="F165" s="35"/>
+      <c r="E165" s="40"/>
+      <c r="F165" s="40"/>
       <c r="G165" s="1"/>
       <c r="H165" s="1"/>
       <c r="I165" s="1"/>
@@ -5354,8 +5678,8 @@
       <c r="B166" s="1"/>
       <c r="C166" s="1"/>
       <c r="D166" s="1"/>
-      <c r="E166" s="35"/>
-      <c r="F166" s="35"/>
+      <c r="E166" s="40"/>
+      <c r="F166" s="40"/>
       <c r="G166" s="1"/>
       <c r="H166" s="1"/>
       <c r="I166" s="1"/>
@@ -5380,8 +5704,8 @@
       <c r="B167" s="1"/>
       <c r="C167" s="1"/>
       <c r="D167" s="1"/>
-      <c r="E167" s="35"/>
-      <c r="F167" s="35"/>
+      <c r="E167" s="40"/>
+      <c r="F167" s="40"/>
       <c r="G167" s="1"/>
       <c r="H167" s="1"/>
       <c r="I167" s="1"/>
@@ -5406,8 +5730,8 @@
       <c r="B168" s="1"/>
       <c r="C168" s="1"/>
       <c r="D168" s="1"/>
-      <c r="E168" s="35"/>
-      <c r="F168" s="35"/>
+      <c r="E168" s="40"/>
+      <c r="F168" s="40"/>
       <c r="G168" s="1"/>
       <c r="H168" s="1"/>
       <c r="I168" s="1"/>
@@ -5432,8 +5756,8 @@
       <c r="B169" s="1"/>
       <c r="C169" s="1"/>
       <c r="D169" s="1"/>
-      <c r="E169" s="35"/>
-      <c r="F169" s="35"/>
+      <c r="E169" s="40"/>
+      <c r="F169" s="40"/>
       <c r="G169" s="1"/>
       <c r="H169" s="1"/>
       <c r="I169" s="1"/>
@@ -5458,8 +5782,8 @@
       <c r="B170" s="1"/>
       <c r="C170" s="1"/>
       <c r="D170" s="1"/>
-      <c r="E170" s="35"/>
-      <c r="F170" s="35"/>
+      <c r="E170" s="40"/>
+      <c r="F170" s="40"/>
       <c r="G170" s="1"/>
       <c r="H170" s="1"/>
       <c r="I170" s="1"/>
@@ -5484,8 +5808,8 @@
       <c r="B171" s="1"/>
       <c r="C171" s="1"/>
       <c r="D171" s="1"/>
-      <c r="E171" s="35"/>
-      <c r="F171" s="35"/>
+      <c r="E171" s="40"/>
+      <c r="F171" s="40"/>
       <c r="G171" s="1"/>
       <c r="H171" s="1"/>
       <c r="I171" s="1"/>
@@ -5510,8 +5834,8 @@
       <c r="B172" s="1"/>
       <c r="C172" s="1"/>
       <c r="D172" s="1"/>
-      <c r="E172" s="35"/>
-      <c r="F172" s="35"/>
+      <c r="E172" s="40"/>
+      <c r="F172" s="40"/>
       <c r="G172" s="1"/>
       <c r="H172" s="1"/>
       <c r="I172" s="1"/>
@@ -5536,8 +5860,8 @@
       <c r="B173" s="1"/>
       <c r="C173" s="1"/>
       <c r="D173" s="1"/>
-      <c r="E173" s="35"/>
-      <c r="F173" s="35"/>
+      <c r="E173" s="40"/>
+      <c r="F173" s="40"/>
       <c r="G173" s="1"/>
       <c r="H173" s="1"/>
       <c r="I173" s="1"/>
@@ -5562,8 +5886,8 @@
       <c r="B174" s="1"/>
       <c r="C174" s="1"/>
       <c r="D174" s="1"/>
-      <c r="E174" s="35"/>
-      <c r="F174" s="35"/>
+      <c r="E174" s="40"/>
+      <c r="F174" s="40"/>
       <c r="G174" s="1"/>
       <c r="H174" s="1"/>
       <c r="I174" s="1"/>
@@ -5588,8 +5912,8 @@
       <c r="B175" s="1"/>
       <c r="C175" s="1"/>
       <c r="D175" s="1"/>
-      <c r="E175" s="35"/>
-      <c r="F175" s="35"/>
+      <c r="E175" s="40"/>
+      <c r="F175" s="40"/>
       <c r="G175" s="1"/>
       <c r="H175" s="1"/>
       <c r="I175" s="1"/>
@@ -5614,8 +5938,8 @@
       <c r="B176" s="1"/>
       <c r="C176" s="1"/>
       <c r="D176" s="1"/>
-      <c r="E176" s="35"/>
-      <c r="F176" s="35"/>
+      <c r="E176" s="40"/>
+      <c r="F176" s="40"/>
       <c r="G176" s="1"/>
       <c r="H176" s="1"/>
       <c r="I176" s="1"/>
@@ -5640,8 +5964,8 @@
       <c r="B177" s="1"/>
       <c r="C177" s="1"/>
       <c r="D177" s="1"/>
-      <c r="E177" s="35"/>
-      <c r="F177" s="35"/>
+      <c r="E177" s="40"/>
+      <c r="F177" s="40"/>
       <c r="G177" s="1"/>
       <c r="H177" s="1"/>
       <c r="I177" s="1"/>
@@ -5666,8 +5990,8 @@
       <c r="B178" s="1"/>
       <c r="C178" s="1"/>
       <c r="D178" s="1"/>
-      <c r="E178" s="35"/>
-      <c r="F178" s="35"/>
+      <c r="E178" s="40"/>
+      <c r="F178" s="40"/>
       <c r="G178" s="1"/>
       <c r="H178" s="1"/>
       <c r="I178" s="1"/>
@@ -5692,8 +6016,8 @@
       <c r="B179" s="1"/>
       <c r="C179" s="1"/>
       <c r="D179" s="1"/>
-      <c r="E179" s="35"/>
-      <c r="F179" s="35"/>
+      <c r="E179" s="40"/>
+      <c r="F179" s="40"/>
       <c r="G179" s="1"/>
       <c r="H179" s="1"/>
       <c r="I179" s="1"/>
@@ -5718,8 +6042,8 @@
       <c r="B180" s="1"/>
       <c r="C180" s="1"/>
       <c r="D180" s="1"/>
-      <c r="E180" s="35"/>
-      <c r="F180" s="35"/>
+      <c r="E180" s="40"/>
+      <c r="F180" s="40"/>
       <c r="G180" s="1"/>
       <c r="H180" s="1"/>
       <c r="I180" s="1"/>
@@ -5744,8 +6068,8 @@
       <c r="B181" s="1"/>
       <c r="C181" s="1"/>
       <c r="D181" s="1"/>
-      <c r="E181" s="35"/>
-      <c r="F181" s="35"/>
+      <c r="E181" s="40"/>
+      <c r="F181" s="40"/>
       <c r="G181" s="1"/>
       <c r="H181" s="1"/>
       <c r="I181" s="1"/>
@@ -5770,8 +6094,8 @@
       <c r="B182" s="1"/>
       <c r="C182" s="1"/>
       <c r="D182" s="1"/>
-      <c r="E182" s="35"/>
-      <c r="F182" s="35"/>
+      <c r="E182" s="40"/>
+      <c r="F182" s="40"/>
       <c r="G182" s="1"/>
       <c r="H182" s="1"/>
       <c r="I182" s="1"/>
@@ -5796,8 +6120,8 @@
       <c r="B183" s="1"/>
       <c r="C183" s="1"/>
       <c r="D183" s="1"/>
-      <c r="E183" s="35"/>
-      <c r="F183" s="35"/>
+      <c r="E183" s="40"/>
+      <c r="F183" s="40"/>
       <c r="G183" s="1"/>
       <c r="H183" s="1"/>
       <c r="I183" s="1"/>
@@ -5822,8 +6146,8 @@
       <c r="B184" s="1"/>
       <c r="C184" s="1"/>
       <c r="D184" s="1"/>
-      <c r="E184" s="35"/>
-      <c r="F184" s="35"/>
+      <c r="E184" s="40"/>
+      <c r="F184" s="40"/>
       <c r="G184" s="1"/>
       <c r="H184" s="1"/>
       <c r="I184" s="1"/>
@@ -5848,8 +6172,8 @@
       <c r="B185" s="1"/>
       <c r="C185" s="1"/>
       <c r="D185" s="1"/>
-      <c r="E185" s="35"/>
-      <c r="F185" s="35"/>
+      <c r="E185" s="40"/>
+      <c r="F185" s="40"/>
       <c r="G185" s="1"/>
       <c r="H185" s="1"/>
       <c r="I185" s="1"/>
@@ -5874,8 +6198,8 @@
       <c r="B186" s="1"/>
       <c r="C186" s="1"/>
       <c r="D186" s="1"/>
-      <c r="E186" s="35"/>
-      <c r="F186" s="35"/>
+      <c r="E186" s="40"/>
+      <c r="F186" s="40"/>
       <c r="G186" s="1"/>
       <c r="H186" s="1"/>
       <c r="I186" s="1"/>
@@ -5900,8 +6224,8 @@
       <c r="B187" s="1"/>
       <c r="C187" s="1"/>
       <c r="D187" s="1"/>
-      <c r="E187" s="35"/>
-      <c r="F187" s="35"/>
+      <c r="E187" s="40"/>
+      <c r="F187" s="40"/>
       <c r="G187" s="1"/>
       <c r="H187" s="1"/>
       <c r="I187" s="1"/>
@@ -5926,8 +6250,8 @@
       <c r="B188" s="1"/>
       <c r="C188" s="1"/>
       <c r="D188" s="1"/>
-      <c r="E188" s="35"/>
-      <c r="F188" s="35"/>
+      <c r="E188" s="40"/>
+      <c r="F188" s="40"/>
       <c r="G188" s="1"/>
       <c r="H188" s="1"/>
       <c r="I188" s="1"/>
@@ -5952,8 +6276,8 @@
       <c r="B189" s="1"/>
       <c r="C189" s="1"/>
       <c r="D189" s="1"/>
-      <c r="E189" s="35"/>
-      <c r="F189" s="35"/>
+      <c r="E189" s="40"/>
+      <c r="F189" s="40"/>
       <c r="G189" s="1"/>
       <c r="H189" s="1"/>
       <c r="I189" s="1"/>
@@ -5978,8 +6302,8 @@
       <c r="B190" s="1"/>
       <c r="C190" s="1"/>
       <c r="D190" s="1"/>
-      <c r="E190" s="35"/>
-      <c r="F190" s="35"/>
+      <c r="E190" s="40"/>
+      <c r="F190" s="40"/>
       <c r="G190" s="1"/>
       <c r="H190" s="1"/>
       <c r="I190" s="1"/>
@@ -6004,8 +6328,8 @@
       <c r="B191" s="1"/>
       <c r="C191" s="1"/>
       <c r="D191" s="1"/>
-      <c r="E191" s="35"/>
-      <c r="F191" s="35"/>
+      <c r="E191" s="40"/>
+      <c r="F191" s="40"/>
       <c r="G191" s="1"/>
       <c r="H191" s="1"/>
       <c r="I191" s="1"/>
@@ -6030,8 +6354,8 @@
       <c r="B192" s="1"/>
       <c r="C192" s="1"/>
       <c r="D192" s="1"/>
-      <c r="E192" s="35"/>
-      <c r="F192" s="35"/>
+      <c r="E192" s="40"/>
+      <c r="F192" s="40"/>
       <c r="G192" s="1"/>
       <c r="H192" s="1"/>
       <c r="I192" s="1"/>
@@ -6056,8 +6380,8 @@
       <c r="B193" s="1"/>
       <c r="C193" s="1"/>
       <c r="D193" s="1"/>
-      <c r="E193" s="35"/>
-      <c r="F193" s="35"/>
+      <c r="E193" s="40"/>
+      <c r="F193" s="40"/>
       <c r="G193" s="1"/>
       <c r="H193" s="1"/>
       <c r="I193" s="1"/>
@@ -6082,8 +6406,8 @@
       <c r="B194" s="1"/>
       <c r="C194" s="1"/>
       <c r="D194" s="1"/>
-      <c r="E194" s="35"/>
-      <c r="F194" s="35"/>
+      <c r="E194" s="40"/>
+      <c r="F194" s="40"/>
       <c r="G194" s="1"/>
       <c r="H194" s="1"/>
       <c r="I194" s="1"/>
@@ -6108,8 +6432,8 @@
       <c r="B195" s="1"/>
       <c r="C195" s="1"/>
       <c r="D195" s="1"/>
-      <c r="E195" s="35"/>
-      <c r="F195" s="35"/>
+      <c r="E195" s="40"/>
+      <c r="F195" s="40"/>
       <c r="G195" s="1"/>
       <c r="H195" s="1"/>
       <c r="I195" s="1"/>
@@ -6134,8 +6458,8 @@
       <c r="B196" s="1"/>
       <c r="C196" s="1"/>
       <c r="D196" s="1"/>
-      <c r="E196" s="35"/>
-      <c r="F196" s="35"/>
+      <c r="E196" s="40"/>
+      <c r="F196" s="40"/>
       <c r="G196" s="1"/>
       <c r="H196" s="1"/>
       <c r="I196" s="1"/>
@@ -6160,8 +6484,8 @@
       <c r="B197" s="1"/>
       <c r="C197" s="1"/>
       <c r="D197" s="1"/>
-      <c r="E197" s="35"/>
-      <c r="F197" s="35"/>
+      <c r="E197" s="40"/>
+      <c r="F197" s="40"/>
       <c r="G197" s="1"/>
       <c r="H197" s="1"/>
       <c r="I197" s="1"/>
@@ -6186,8 +6510,8 @@
       <c r="B198" s="1"/>
       <c r="C198" s="1"/>
       <c r="D198" s="1"/>
-      <c r="E198" s="35"/>
-      <c r="F198" s="35"/>
+      <c r="E198" s="40"/>
+      <c r="F198" s="40"/>
       <c r="G198" s="1"/>
       <c r="H198" s="1"/>
       <c r="I198" s="1"/>
@@ -6212,8 +6536,8 @@
       <c r="B199" s="1"/>
       <c r="C199" s="1"/>
       <c r="D199" s="1"/>
-      <c r="E199" s="35"/>
-      <c r="F199" s="35"/>
+      <c r="E199" s="40"/>
+      <c r="F199" s="40"/>
       <c r="G199" s="1"/>
       <c r="H199" s="1"/>
       <c r="I199" s="1"/>
@@ -6238,8 +6562,8 @@
       <c r="B200" s="1"/>
       <c r="C200" s="1"/>
       <c r="D200" s="1"/>
-      <c r="E200" s="35"/>
-      <c r="F200" s="35"/>
+      <c r="E200" s="40"/>
+      <c r="F200" s="40"/>
       <c r="G200" s="1"/>
       <c r="H200" s="1"/>
       <c r="I200" s="1"/>
@@ -6264,8 +6588,8 @@
       <c r="B201" s="1"/>
       <c r="C201" s="1"/>
       <c r="D201" s="1"/>
-      <c r="E201" s="35"/>
-      <c r="F201" s="35"/>
+      <c r="E201" s="40"/>
+      <c r="F201" s="40"/>
       <c r="G201" s="1"/>
       <c r="H201" s="1"/>
       <c r="I201" s="1"/>
@@ -6290,8 +6614,8 @@
       <c r="B202" s="1"/>
       <c r="C202" s="1"/>
       <c r="D202" s="1"/>
-      <c r="E202" s="35"/>
-      <c r="F202" s="35"/>
+      <c r="E202" s="40"/>
+      <c r="F202" s="40"/>
       <c r="G202" s="1"/>
       <c r="H202" s="1"/>
       <c r="I202" s="1"/>
@@ -6316,8 +6640,8 @@
       <c r="B203" s="1"/>
       <c r="C203" s="1"/>
       <c r="D203" s="1"/>
-      <c r="E203" s="35"/>
-      <c r="F203" s="35"/>
+      <c r="E203" s="40"/>
+      <c r="F203" s="40"/>
       <c r="G203" s="1"/>
       <c r="H203" s="1"/>
       <c r="I203" s="1"/>
@@ -6342,8 +6666,8 @@
       <c r="B204" s="1"/>
       <c r="C204" s="1"/>
       <c r="D204" s="1"/>
-      <c r="E204" s="35"/>
-      <c r="F204" s="35"/>
+      <c r="E204" s="40"/>
+      <c r="F204" s="40"/>
       <c r="G204" s="1"/>
       <c r="H204" s="1"/>
       <c r="I204" s="1"/>
@@ -6368,8 +6692,8 @@
       <c r="B205" s="1"/>
       <c r="C205" s="1"/>
       <c r="D205" s="1"/>
-      <c r="E205" s="35"/>
-      <c r="F205" s="35"/>
+      <c r="E205" s="40"/>
+      <c r="F205" s="40"/>
       <c r="G205" s="1"/>
       <c r="H205" s="1"/>
       <c r="I205" s="1"/>
@@ -6394,8 +6718,8 @@
       <c r="B206" s="1"/>
       <c r="C206" s="1"/>
       <c r="D206" s="1"/>
-      <c r="E206" s="35"/>
-      <c r="F206" s="35"/>
+      <c r="E206" s="40"/>
+      <c r="F206" s="40"/>
       <c r="G206" s="1"/>
       <c r="H206" s="1"/>
       <c r="I206" s="1"/>
@@ -6420,8 +6744,8 @@
       <c r="B207" s="1"/>
       <c r="C207" s="1"/>
       <c r="D207" s="1"/>
-      <c r="E207" s="35"/>
-      <c r="F207" s="35"/>
+      <c r="E207" s="40"/>
+      <c r="F207" s="40"/>
       <c r="G207" s="1"/>
       <c r="H207" s="1"/>
       <c r="I207" s="1"/>
@@ -6446,8 +6770,8 @@
       <c r="B208" s="1"/>
       <c r="C208" s="1"/>
       <c r="D208" s="1"/>
-      <c r="E208" s="35"/>
-      <c r="F208" s="35"/>
+      <c r="E208" s="40"/>
+      <c r="F208" s="40"/>
       <c r="G208" s="1"/>
       <c r="H208" s="1"/>
       <c r="I208" s="1"/>
@@ -6472,8 +6796,8 @@
       <c r="B209" s="1"/>
       <c r="C209" s="1"/>
       <c r="D209" s="1"/>
-      <c r="E209" s="35"/>
-      <c r="F209" s="35"/>
+      <c r="E209" s="40"/>
+      <c r="F209" s="40"/>
       <c r="G209" s="1"/>
       <c r="H209" s="1"/>
       <c r="I209" s="1"/>
@@ -6498,8 +6822,8 @@
       <c r="B210" s="1"/>
       <c r="C210" s="1"/>
       <c r="D210" s="1"/>
-      <c r="E210" s="35"/>
-      <c r="F210" s="35"/>
+      <c r="E210" s="40"/>
+      <c r="F210" s="40"/>
       <c r="G210" s="1"/>
       <c r="H210" s="1"/>
       <c r="I210" s="1"/>
@@ -6524,8 +6848,8 @@
       <c r="B211" s="1"/>
       <c r="C211" s="1"/>
       <c r="D211" s="1"/>
-      <c r="E211" s="35"/>
-      <c r="F211" s="35"/>
+      <c r="E211" s="40"/>
+      <c r="F211" s="40"/>
       <c r="G211" s="1"/>
       <c r="H211" s="1"/>
       <c r="I211" s="1"/>
@@ -6550,8 +6874,8 @@
       <c r="B212" s="1"/>
       <c r="C212" s="1"/>
       <c r="D212" s="1"/>
-      <c r="E212" s="35"/>
-      <c r="F212" s="35"/>
+      <c r="E212" s="40"/>
+      <c r="F212" s="40"/>
       <c r="G212" s="1"/>
       <c r="H212" s="1"/>
       <c r="I212" s="1"/>
@@ -6576,8 +6900,8 @@
       <c r="B213" s="1"/>
       <c r="C213" s="1"/>
       <c r="D213" s="1"/>
-      <c r="E213" s="35"/>
-      <c r="F213" s="35"/>
+      <c r="E213" s="40"/>
+      <c r="F213" s="40"/>
       <c r="G213" s="1"/>
       <c r="H213" s="1"/>
       <c r="I213" s="1"/>
@@ -6602,8 +6926,8 @@
       <c r="B214" s="1"/>
       <c r="C214" s="1"/>
       <c r="D214" s="1"/>
-      <c r="E214" s="35"/>
-      <c r="F214" s="35"/>
+      <c r="E214" s="40"/>
+      <c r="F214" s="40"/>
       <c r="G214" s="1"/>
       <c r="H214" s="1"/>
       <c r="I214" s="1"/>
@@ -6628,8 +6952,8 @@
       <c r="B215" s="1"/>
       <c r="C215" s="1"/>
       <c r="D215" s="1"/>
-      <c r="E215" s="35"/>
-      <c r="F215" s="35"/>
+      <c r="E215" s="40"/>
+      <c r="F215" s="40"/>
       <c r="G215" s="1"/>
       <c r="H215" s="1"/>
       <c r="I215" s="1"/>
@@ -6654,8 +6978,8 @@
       <c r="B216" s="1"/>
       <c r="C216" s="1"/>
       <c r="D216" s="1"/>
-      <c r="E216" s="35"/>
-      <c r="F216" s="35"/>
+      <c r="E216" s="40"/>
+      <c r="F216" s="40"/>
       <c r="G216" s="1"/>
       <c r="H216" s="1"/>
       <c r="I216" s="1"/>
@@ -6680,8 +7004,8 @@
       <c r="B217" s="1"/>
       <c r="C217" s="1"/>
       <c r="D217" s="1"/>
-      <c r="E217" s="35"/>
-      <c r="F217" s="35"/>
+      <c r="E217" s="1"/>
+      <c r="F217" s="1"/>
       <c r="G217" s="1"/>
       <c r="H217" s="1"/>
       <c r="I217" s="1"/>
@@ -26955,62 +27279,24 @@
       <c r="W996" s="1"/>
       <c r="X996" s="1"/>
     </row>
-    <row r="997" ht="12.75" customHeight="1">
-      <c r="A997" s="1"/>
-      <c r="B997" s="1"/>
-      <c r="C997" s="1"/>
-      <c r="D997" s="1"/>
-      <c r="E997" s="1"/>
-      <c r="F997" s="1"/>
-      <c r="G997" s="1"/>
-      <c r="H997" s="1"/>
-      <c r="I997" s="1"/>
-      <c r="J997" s="1"/>
-      <c r="K997" s="1"/>
-      <c r="L997" s="1"/>
-      <c r="M997" s="1"/>
-      <c r="N997" s="1"/>
-      <c r="O997" s="1"/>
-      <c r="P997" s="1"/>
-      <c r="Q997" s="1"/>
-      <c r="R997" s="1"/>
-      <c r="S997" s="1"/>
-      <c r="T997" s="1"/>
-      <c r="U997" s="1"/>
-      <c r="V997" s="1"/>
-      <c r="W997" s="1"/>
-      <c r="X997" s="1"/>
-    </row>
   </sheetData>
-  <mergeCells count="217">
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="M26:N26"/>
-    <mergeCell ref="O26:P26"/>
-    <mergeCell ref="Q26:R26"/>
-    <mergeCell ref="S26:T26"/>
-    <mergeCell ref="G27:H27"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="M27:N27"/>
-    <mergeCell ref="O27:P27"/>
-    <mergeCell ref="Q27:R27"/>
-    <mergeCell ref="S27:T27"/>
-    <mergeCell ref="G28:H28"/>
-    <mergeCell ref="I28:J28"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="O28:P28"/>
-    <mergeCell ref="Q28:R28"/>
-    <mergeCell ref="S28:T28"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="O29:P29"/>
-    <mergeCell ref="Q29:R29"/>
-    <mergeCell ref="S29:T29"/>
+  <mergeCells count="210">
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="Q21:R21"/>
+    <mergeCell ref="S21:T21"/>
+    <mergeCell ref="S19:T19"/>
+    <mergeCell ref="Q19:R19"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="I20:J20"/>
     <mergeCell ref="G30:H30"/>
     <mergeCell ref="I30:J30"/>
     <mergeCell ref="K30:L30"/>
@@ -27039,6 +27325,31 @@
     <mergeCell ref="O33:P33"/>
     <mergeCell ref="Q33:R33"/>
     <mergeCell ref="S33:T33"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="O17:P17"/>
+    <mergeCell ref="S17:T17"/>
+    <mergeCell ref="Q17:R17"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="Q18:R18"/>
+    <mergeCell ref="S18:T18"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="Q20:R20"/>
+    <mergeCell ref="S20:T20"/>
+    <mergeCell ref="G35:H35"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="M35:N35"/>
+    <mergeCell ref="O35:P35"/>
+    <mergeCell ref="Q35:R35"/>
+    <mergeCell ref="S35:T35"/>
     <mergeCell ref="G34:H34"/>
     <mergeCell ref="I34:J34"/>
     <mergeCell ref="K34:L34"/>
@@ -27046,13 +27357,35 @@
     <mergeCell ref="O34:P34"/>
     <mergeCell ref="Q34:R34"/>
     <mergeCell ref="S34:T34"/>
-    <mergeCell ref="G35:H35"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="K35:L35"/>
-    <mergeCell ref="M35:N35"/>
-    <mergeCell ref="O35:P35"/>
-    <mergeCell ref="Q35:R35"/>
-    <mergeCell ref="S35:T35"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="K12:L12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="O12:P12"/>
+    <mergeCell ref="Q12:R12"/>
+    <mergeCell ref="S12:T12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="K13:L13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="O13:P13"/>
+    <mergeCell ref="Q13:R13"/>
+    <mergeCell ref="S13:T13"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="K14:L14"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="O14:P14"/>
+    <mergeCell ref="Q14:R14"/>
+    <mergeCell ref="S14:T14"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="Q15:R15"/>
+    <mergeCell ref="S15:T15"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="I6:J6"/>
     <mergeCell ref="K6:L6"/>
@@ -27095,41 +27428,6 @@
     <mergeCell ref="O11:P11"/>
     <mergeCell ref="Q11:R11"/>
     <mergeCell ref="S11:T11"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="I36:J36"/>
-    <mergeCell ref="K36:L36"/>
-    <mergeCell ref="M36:N36"/>
-    <mergeCell ref="O36:P36"/>
-    <mergeCell ref="Q36:R36"/>
-    <mergeCell ref="S36:T36"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="K12:L12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="O12:P12"/>
-    <mergeCell ref="Q12:R12"/>
-    <mergeCell ref="S12:T12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="K13:L13"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="O13:P13"/>
-    <mergeCell ref="Q13:R13"/>
-    <mergeCell ref="S13:T13"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="K14:L14"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="O14:P14"/>
-    <mergeCell ref="Q14:R14"/>
-    <mergeCell ref="S14:T14"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="S15:T15"/>
     <mergeCell ref="G16:H16"/>
     <mergeCell ref="I16:J16"/>
     <mergeCell ref="K16:L16"/>
@@ -27137,41 +27435,6 @@
     <mergeCell ref="O16:P16"/>
     <mergeCell ref="Q16:R16"/>
     <mergeCell ref="S16:T16"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="O17:P17"/>
-    <mergeCell ref="Q17:R17"/>
-    <mergeCell ref="S17:T17"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="O18:P18"/>
-    <mergeCell ref="Q18:R18"/>
-    <mergeCell ref="S18:T18"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="O19:P19"/>
-    <mergeCell ref="Q19:R19"/>
-    <mergeCell ref="S19:T19"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="O20:P20"/>
-    <mergeCell ref="Q20:R20"/>
-    <mergeCell ref="S20:T20"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="Q21:R21"/>
-    <mergeCell ref="S21:T21"/>
     <mergeCell ref="G22:H22"/>
     <mergeCell ref="I22:J22"/>
     <mergeCell ref="K22:L22"/>
@@ -27200,6 +27463,34 @@
     <mergeCell ref="O25:P25"/>
     <mergeCell ref="Q25:R25"/>
     <mergeCell ref="S25:T25"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="M26:N26"/>
+    <mergeCell ref="O26:P26"/>
+    <mergeCell ref="Q26:R26"/>
+    <mergeCell ref="S26:T26"/>
+    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="M27:N27"/>
+    <mergeCell ref="O27:P27"/>
+    <mergeCell ref="Q27:R27"/>
+    <mergeCell ref="S27:T27"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="O28:P28"/>
+    <mergeCell ref="Q28:R28"/>
+    <mergeCell ref="S28:T28"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="O29:P29"/>
+    <mergeCell ref="Q29:R29"/>
+    <mergeCell ref="S29:T29"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.0" footer="0.0" header="0.0" left="0.0" right="0.0" top="0.984251968503937"/>

</xml_diff>